<commit_message>
describe thworkflow with GIFs
</commit_message>
<xml_diff>
--- a/pin_points_inventor.xlsx
+++ b/pin_points_inventor.xlsx
@@ -23,1861 +23,1817 @@
     </row>
     <row r="2">
       <c r="A2">
-        <v>3.19355908</v>
+        <v>2.09455331</v>
       </c>
       <c r="B2">
-        <v>19.65709983</v>
+        <v>19.89001876</v>
       </c>
       <c r="C2">
-        <v>1.8438022</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3">
-        <v>0</v>
+        <v>-2.18118094</v>
       </c>
       <c r="B3">
-        <v>19.65709983</v>
+        <v>19.78003753</v>
       </c>
       <c r="C3">
-        <v>3.68760439</v>
+        <v>1.99814041</v>
       </c>
     </row>
     <row r="4">
       <c r="A4">
-        <v>-3.19355908</v>
+        <v>0.31629372</v>
       </c>
       <c r="B4">
-        <v>19.65709983</v>
+        <v>19.67005629</v>
       </c>
       <c r="C4">
-        <v>1.8438022</v>
+        <v>-3.60400385</v>
       </c>
     </row>
     <row r="5">
       <c r="A5">
-        <v>-3.19355908</v>
+        <v>2.53825232</v>
       </c>
       <c r="B5">
-        <v>19.65709983</v>
+        <v>19.56007506</v>
       </c>
       <c r="C5">
-        <v>-1.8438022</v>
+        <v>3.31070067</v>
       </c>
     </row>
     <row r="6">
       <c r="A6">
-        <v>0</v>
+        <v>-4.58646629</v>
       </c>
       <c r="B6">
-        <v>19.65709983</v>
+        <v>19.45009382</v>
       </c>
       <c r="C6">
-        <v>-3.68760439</v>
+        <v>-0.81128131</v>
       </c>
     </row>
     <row r="7">
       <c r="A7">
-        <v>3.19355908</v>
+        <v>4.2990177</v>
       </c>
       <c r="B7">
-        <v>19.65709983</v>
+        <v>19.34011259</v>
       </c>
       <c r="C7">
-        <v>-1.8438022</v>
+        <v>-2.73468316</v>
       </c>
     </row>
     <row r="8">
       <c r="A8">
-        <v>7.24876077</v>
+        <v>-1.42669155</v>
       </c>
       <c r="B8">
-        <v>18.64015739</v>
+        <v>19.23013135</v>
       </c>
       <c r="C8">
-        <v>0</v>
+        <v>5.30722145</v>
       </c>
     </row>
     <row r="9">
       <c r="A9">
-        <v>6.0980456</v>
+        <v>-2.70406966</v>
       </c>
       <c r="B9">
-        <v>18.64015739</v>
+        <v>19.12015011</v>
       </c>
       <c r="C9">
-        <v>3.91897595</v>
+        <v>-5.20652158</v>
       </c>
     </row>
     <row r="10">
       <c r="A10">
-        <v>3.01124405</v>
+        <v>5.83691859</v>
       </c>
       <c r="B10">
-        <v>18.64015739</v>
+        <v>19.01016888</v>
       </c>
       <c r="C10">
-        <v>6.59370472</v>
+        <v>2.13163331</v>
       </c>
     </row>
     <row r="11">
       <c r="A11">
-        <v>-1.03160622</v>
+        <v>-6.04601894</v>
       </c>
       <c r="B11">
-        <v>18.64015739</v>
+        <v>18.90018764</v>
       </c>
       <c r="C11">
-        <v>7.17497883</v>
+        <v>2.49570873</v>
       </c>
     </row>
     <row r="12">
       <c r="A12">
-        <v>-4.7469288</v>
+        <v>2.90351965</v>
       </c>
       <c r="B12">
-        <v>18.64015739</v>
+        <v>18.79020641</v>
       </c>
       <c r="C12">
-        <v>5.47824786</v>
+        <v>-6.20465284</v>
       </c>
     </row>
     <row r="13">
       <c r="A13">
-        <v>-6.95513502</v>
+        <v>2.13834473</v>
       </c>
       <c r="B13">
-        <v>18.64015739</v>
+        <v>18.68022517</v>
       </c>
       <c r="C13">
-        <v>2.0422119</v>
+        <v>6.81737995</v>
       </c>
     </row>
     <row r="14">
       <c r="A14">
-        <v>-6.95513502</v>
+        <v>-6.42509131</v>
       </c>
       <c r="B14">
-        <v>18.64015739</v>
+        <v>18.57024393</v>
       </c>
       <c r="C14">
-        <v>-2.0422119</v>
+        <v>-3.72347175</v>
       </c>
     </row>
     <row r="15">
       <c r="A15">
-        <v>-4.7469288</v>
+        <v>7.51588028</v>
       </c>
       <c r="B15">
-        <v>18.64015739</v>
+        <v>18.4602627</v>
       </c>
       <c r="C15">
-        <v>-5.47824786</v>
+        <v>-1.6523452</v>
       </c>
     </row>
     <row r="16">
       <c r="A16">
-        <v>-1.03160622</v>
+        <v>-4.57461759</v>
       </c>
       <c r="B16">
-        <v>18.64015739</v>
+        <v>18.35028146</v>
       </c>
       <c r="C16">
-        <v>-7.17497883</v>
+        <v>6.50692278</v>
       </c>
     </row>
     <row r="17">
       <c r="A17">
-        <v>3.01124405</v>
+        <v>-1.05419072</v>
       </c>
       <c r="B17">
-        <v>18.64015739</v>
+        <v>18.24030023</v>
       </c>
       <c r="C17">
-        <v>-6.59370472</v>
+        <v>-8.13511706</v>
       </c>
     </row>
     <row r="18">
       <c r="A18">
-        <v>6.0980456</v>
+        <v>6.45626131</v>
       </c>
       <c r="B18">
-        <v>18.64015739</v>
+        <v>18.13031899</v>
       </c>
       <c r="C18">
-        <v>-3.91897595</v>
+        <v>5.44134387</v>
       </c>
     </row>
     <row r="19">
       <c r="A19">
-        <v>10.38152984</v>
+        <v>-8.66827165</v>
       </c>
       <c r="B19">
-        <v>16.98404363</v>
+        <v>18.02033776</v>
       </c>
       <c r="C19">
-        <v>1.94064426</v>
+        <v>0.35846025</v>
       </c>
     </row>
     <row r="20">
       <c r="A20">
-        <v>8.97944671</v>
+        <v>6.30894532</v>
       </c>
       <c r="B20">
-        <v>16.98404363</v>
+        <v>17.91035652</v>
       </c>
       <c r="C20">
-        <v>5.55983802</v>
+        <v>-6.27824324</v>
       </c>
     </row>
     <row r="21">
       <c r="A21">
-        <v>6.36463954</v>
+        <v>-0.42119568</v>
       </c>
       <c r="B21">
-        <v>16.98404363</v>
+        <v>17.80037528</v>
       </c>
       <c r="C21">
-        <v>8.42814484</v>
+        <v>9.10874492</v>
       </c>
     </row>
     <row r="22">
       <c r="A22">
-        <v>2.89025254</v>
+        <v>-5.97785266</v>
       </c>
       <c r="B22">
-        <v>16.98404363</v>
+        <v>17.69039405</v>
       </c>
       <c r="C22">
-        <v>10.158184</v>
+        <v>-7.16346536</v>
       </c>
     </row>
     <row r="23">
       <c r="A23">
-        <v>-0.97447909</v>
+        <v>9.45051518</v>
       </c>
       <c r="B23">
-        <v>16.98404363</v>
+        <v>17.58041281</v>
       </c>
       <c r="C23">
-        <v>10.51630413</v>
+        <v>1.27155345</v>
       </c>
     </row>
     <row r="24">
       <c r="A24">
-        <v>-4.70760191</v>
+        <v>-7.99163751</v>
       </c>
       <c r="B24">
-        <v>16.98404363</v>
+        <v>17.47043158</v>
       </c>
       <c r="C24">
-        <v>9.4541391</v>
+        <v>5.56037323</v>
       </c>
     </row>
     <row r="25">
       <c r="A25">
-        <v>-7.80493701</v>
+        <v>2.179559</v>
       </c>
       <c r="B25">
-        <v>16.98404363</v>
+        <v>17.36045034</v>
       </c>
       <c r="C25">
-        <v>7.11514021</v>
+        <v>-9.6883583</v>
       </c>
     </row>
     <row r="26">
       <c r="A26">
-        <v>-9.84817212</v>
+        <v>5.03164033</v>
       </c>
       <c r="B26">
-        <v>16.98404363</v>
+        <v>17.2504691</v>
       </c>
       <c r="C26">
-        <v>3.8152022</v>
+        <v>8.78088328</v>
       </c>
     </row>
     <row r="27">
       <c r="A27">
-        <v>-10.56135701</v>
+        <v>-9.81799138</v>
       </c>
       <c r="B27">
-        <v>16.98404363</v>
+        <v>17.14048787</v>
       </c>
       <c r="C27">
-        <v>0</v>
+        <v>-3.13220703</v>
       </c>
     </row>
     <row r="28">
       <c r="A28">
-        <v>-9.84817212</v>
+        <v>9.51934229</v>
       </c>
       <c r="B28">
-        <v>16.98404363</v>
+        <v>17.03050663</v>
       </c>
       <c r="C28">
-        <v>-3.8152022</v>
+        <v>-4.39817759</v>
       </c>
     </row>
     <row r="29">
       <c r="A29">
-        <v>-7.80493701</v>
+        <v>-4.11650146</v>
       </c>
       <c r="B29">
-        <v>16.98404363</v>
+        <v>16.9205254</v>
       </c>
       <c r="C29">
-        <v>-7.11514021</v>
+        <v>9.83616979</v>
       </c>
     </row>
     <row r="30">
       <c r="A30">
-        <v>-4.70760191</v>
+        <v>-3.66726133</v>
       </c>
       <c r="B30">
-        <v>16.98404363</v>
+        <v>16.81054416</v>
       </c>
       <c r="C30">
-        <v>-9.4541391</v>
+        <v>-10.19592072</v>
       </c>
     </row>
     <row r="31">
       <c r="A31">
-        <v>-0.97447909</v>
+        <v>9.74075255</v>
       </c>
       <c r="B31">
-        <v>16.98404363</v>
+        <v>16.70056293</v>
       </c>
       <c r="C31">
-        <v>-10.51630413</v>
+        <v>5.11946655</v>
       </c>
     </row>
     <row r="32">
       <c r="A32">
-        <v>2.89025254</v>
+        <v>-10.80034937</v>
       </c>
       <c r="B32">
-        <v>16.98404363</v>
+        <v>16.59058169</v>
       </c>
       <c r="C32">
-        <v>-10.158184</v>
+        <v>2.84693743</v>
       </c>
     </row>
     <row r="33">
       <c r="A33">
-        <v>6.36463954</v>
+        <v>6.12819059</v>
       </c>
       <c r="B33">
-        <v>16.98404363</v>
+        <v>16.48060045</v>
       </c>
       <c r="C33">
-        <v>-8.42814484</v>
+        <v>-9.5307444</v>
       </c>
     </row>
     <row r="34">
       <c r="A34">
-        <v>8.97944671</v>
+        <v>1.9460049</v>
       </c>
       <c r="B34">
-        <v>16.98404363</v>
+        <v>16.37061922</v>
       </c>
       <c r="C34">
-        <v>-5.55983802</v>
+        <v>11.32324562</v>
       </c>
     </row>
     <row r="35">
       <c r="A35">
-        <v>10.38152984</v>
+        <v>-9.20631895</v>
       </c>
       <c r="B35">
-        <v>16.98404363</v>
+        <v>16.26063798</v>
       </c>
       <c r="C35">
-        <v>-1.94064426</v>
+        <v>-7.12989086</v>
       </c>
     </row>
     <row r="36">
       <c r="A36">
-        <v>13.51180415</v>
+        <v>11.75617536</v>
       </c>
       <c r="B36">
-        <v>14.74554674</v>
+        <v>16.15065675</v>
       </c>
       <c r="C36">
-        <v>0</v>
+        <v>-0.9739751</v>
       </c>
     </row>
     <row r="37">
       <c r="A37">
-        <v>12.91151261</v>
+        <v>-8.11199233</v>
       </c>
       <c r="B37">
-        <v>14.74554674</v>
+        <v>16.04067551</v>
       </c>
       <c r="C37">
-        <v>3.98267419</v>
+        <v>8.76882601</v>
       </c>
     </row>
     <row r="38">
       <c r="A38">
-        <v>11.1639765</v>
+        <v>0.05898742</v>
       </c>
       <c r="B38">
-        <v>14.74554674</v>
+        <v>15.93069427</v>
       </c>
       <c r="C38">
-        <v>7.6114703</v>
+        <v>-12.09171205</v>
       </c>
     </row>
     <row r="39">
       <c r="A39">
-        <v>8.42447209</v>
+        <v>8.22078448</v>
       </c>
       <c r="B39">
-        <v>14.74554674</v>
+        <v>15.82071304</v>
       </c>
       <c r="C39">
-        <v>10.56395387</v>
+        <v>9.06221504</v>
       </c>
     </row>
     <row r="40">
       <c r="A40">
-        <v>4.93641637</v>
+        <v>-12.32349083</v>
       </c>
       <c r="B40">
-        <v>14.74554674</v>
+        <v>15.7107318</v>
       </c>
       <c r="C40">
-        <v>12.57778378</v>
+        <v>-1.14213836</v>
       </c>
     </row>
     <row r="41">
       <c r="A41">
-        <v>1.00973839</v>
+        <v>9.96866634</v>
       </c>
       <c r="B41">
-        <v>14.74554674</v>
+        <v>15.60075057</v>
       </c>
       <c r="C41">
-        <v>13.47402241</v>
+        <v>-7.56586235</v>
       </c>
     </row>
     <row r="42">
       <c r="A42">
-        <v>-3.00665928</v>
+        <v>-2.26423829</v>
       </c>
       <c r="B42">
-        <v>14.74554674</v>
+        <v>15.49076933</v>
       </c>
       <c r="C42">
-        <v>13.17303501</v>
+        <v>12.44625608</v>
       </c>
     </row>
     <row r="43">
       <c r="A43">
-        <v>-6.75590208</v>
+        <v>-6.80884453</v>
       </c>
       <c r="B43">
-        <v>14.74554674</v>
+        <v>15.3807881</v>
       </c>
       <c r="C43">
-        <v>11.70156565</v>
+        <v>-10.81993502</v>
       </c>
     </row>
     <row r="44">
       <c r="A44">
-        <v>-9.90485333</v>
+        <v>12.45590133</v>
       </c>
       <c r="B44">
-        <v>14.74554674</v>
+        <v>15.27080686</v>
       </c>
       <c r="C44">
-        <v>9.19036082</v>
+        <v>3.41364615</v>
       </c>
     </row>
     <row r="45">
       <c r="A45">
-        <v>-12.17371489</v>
+        <v>-11.60518511</v>
       </c>
       <c r="B45">
-        <v>14.74554674</v>
+        <v>15.16082562</v>
       </c>
       <c r="C45">
-        <v>5.86255211</v>
+        <v>5.95558939</v>
       </c>
     </row>
     <row r="46">
       <c r="A46">
-        <v>-13.36088846</v>
+        <v>4.57841945</v>
       </c>
       <c r="B46">
-        <v>14.74554674</v>
+        <v>15.05084439</v>
       </c>
       <c r="C46">
-        <v>2.01382991</v>
+        <v>-12.34950034</v>
       </c>
     </row>
     <row r="47">
       <c r="A47">
-        <v>-13.36088846</v>
+        <v>5.0129747</v>
       </c>
       <c r="B47">
-        <v>14.74554674</v>
+        <v>14.94086315</v>
       </c>
       <c r="C47">
-        <v>-2.01382991</v>
+        <v>12.31424756</v>
       </c>
     </row>
     <row r="48">
       <c r="A48">
-        <v>-12.17371489</v>
+        <v>-12.12532896</v>
       </c>
       <c r="B48">
-        <v>14.74554674</v>
+        <v>14.83088192</v>
       </c>
       <c r="C48">
-        <v>-5.86255211</v>
+        <v>-5.74641968</v>
       </c>
     </row>
     <row r="49">
       <c r="A49">
-        <v>-9.90485333</v>
+        <v>12.93770803</v>
       </c>
       <c r="B49">
-        <v>14.74554674</v>
+        <v>14.72090068</v>
       </c>
       <c r="C49">
-        <v>-9.19036082</v>
+        <v>-3.98883366</v>
       </c>
     </row>
     <row r="50">
       <c r="A50">
-        <v>-6.75590208</v>
+        <v>-6.90542119</v>
       </c>
       <c r="B50">
-        <v>14.74554674</v>
+        <v>14.61091945</v>
       </c>
       <c r="C50">
-        <v>-11.70156565</v>
+        <v>11.78287703</v>
       </c>
     </row>
     <row r="51">
       <c r="A51">
-        <v>-3.00665928</v>
+        <v>-2.8918819</v>
       </c>
       <c r="B51">
-        <v>14.74554674</v>
+        <v>14.50093821</v>
       </c>
       <c r="C51">
-        <v>-13.17303501</v>
+        <v>-13.46698965</v>
       </c>
     </row>
     <row r="52">
       <c r="A52">
-        <v>1.00973839</v>
+        <v>11.32285003</v>
       </c>
       <c r="B52">
-        <v>14.74554674</v>
+        <v>14.39095697</v>
       </c>
       <c r="C52">
-        <v>-13.47402241</v>
+        <v>8.04322228</v>
       </c>
     </row>
     <row r="53">
       <c r="A53">
-        <v>4.93641637</v>
+        <v>-13.89442942</v>
       </c>
       <c r="B53">
-        <v>14.74554674</v>
+        <v>14.28097574</v>
       </c>
       <c r="C53">
-        <v>-12.57778378</v>
+        <v>1.73163598</v>
       </c>
     </row>
     <row r="54">
       <c r="A54">
-        <v>8.42447209</v>
+        <v>9.14775706</v>
       </c>
       <c r="B54">
-        <v>14.74554674</v>
+        <v>14.1709945</v>
       </c>
       <c r="C54">
-        <v>-10.56395387</v>
+        <v>-10.74716035</v>
       </c>
     </row>
     <row r="55">
       <c r="A55">
-        <v>11.1639765</v>
+        <v>0.5183245</v>
       </c>
       <c r="B55">
-        <v>14.74554674</v>
+        <v>14.06101327</v>
       </c>
       <c r="C55">
-        <v>-7.6114703</v>
+        <v>14.21334745</v>
       </c>
     </row>
     <row r="56">
       <c r="A56">
-        <v>12.91151261</v>
+        <v>-10.0589081</v>
       </c>
       <c r="B56">
-        <v>14.74554674</v>
+        <v>13.95103203</v>
       </c>
       <c r="C56">
-        <v>-3.98267419</v>
+        <v>-10.20720692</v>
       </c>
     </row>
     <row r="57">
       <c r="A57">
-        <v>15.87277495</v>
+        <v>14.41810799</v>
       </c>
       <c r="B57">
-        <v>12.0014248</v>
+        <v>13.84105079</v>
       </c>
       <c r="C57">
-        <v>2.00519779</v>
+        <v>0.73720755</v>
       </c>
     </row>
     <row r="58">
       <c r="A58">
-        <v>14.87543012</v>
+        <v>-11.21011038</v>
       </c>
       <c r="B58">
-        <v>12.0014248</v>
+        <v>13.73106956</v>
       </c>
       <c r="C58">
-        <v>5.88959943</v>
+        <v>9.26235144</v>
       </c>
     </row>
     <row r="59">
       <c r="A59">
-        <v>12.94340732</v>
+        <v>2.02360023</v>
       </c>
       <c r="B59">
-        <v>12.0014248</v>
+        <v>13.62108832</v>
       </c>
       <c r="C59">
-        <v>9.40393587</v>
+        <v>-14.50417164</v>
       </c>
     </row>
     <row r="60">
       <c r="A60">
-        <v>10.19810262</v>
+        <v>8.36286672</v>
       </c>
       <c r="B60">
-        <v>12.0014248</v>
+        <v>13.51110709</v>
       </c>
       <c r="C60">
-        <v>12.32738844</v>
+        <v>12.14547016</v>
       </c>
     </row>
     <row r="61">
       <c r="A61">
-        <v>6.81201364</v>
+        <v>-14.46813811</v>
       </c>
       <c r="B61">
-        <v>12.0014248</v>
+        <v>13.40112585</v>
       </c>
       <c r="C61">
-        <v>14.47626585</v>
+        <v>-3.32908477</v>
       </c>
     </row>
     <row r="62">
       <c r="A62">
-        <v>2.99790078</v>
+        <v>13.00285654</v>
       </c>
       <c r="B62">
-        <v>12.0014248</v>
+        <v>13.29114462</v>
       </c>
       <c r="C62">
-        <v>15.71554624</v>
+        <v>-7.36689871</v>
       </c>
     </row>
     <row r="63">
       <c r="A63">
-        <v>-1.00458121</v>
+        <v>-4.6415937</v>
       </c>
       <c r="B63">
-        <v>12.0014248</v>
+        <v>13.18116338</v>
       </c>
       <c r="C63">
-        <v>15.96736107</v>
+        <v>14.307779</v>
       </c>
     </row>
     <row r="64">
       <c r="A64">
-        <v>-4.94394166</v>
+        <v>-6.28190121</v>
       </c>
       <c r="B64">
-        <v>12.0014248</v>
+        <v>13.07118214</v>
       </c>
       <c r="C64">
-        <v>15.21588787</v>
+        <v>-13.77250575</v>
       </c>
     </row>
     <row r="65">
       <c r="A65">
-        <v>-8.57265608</v>
+        <v>14.02206024</v>
       </c>
       <c r="B65">
-        <v>12.0014248</v>
+        <v>12.96120091</v>
       </c>
       <c r="C65">
-        <v>13.50834448</v>
+        <v>5.94887364</v>
       </c>
     </row>
     <row r="66">
       <c r="A66">
-        <v>-11.66271899</v>
+        <v>-14.44541267</v>
       </c>
       <c r="B66">
-        <v>12.0014248</v>
+        <v>12.85121967</v>
       </c>
       <c r="C66">
-        <v>10.95202212</v>
+        <v>5.11626874</v>
       </c>
     </row>
     <row r="67">
       <c r="A67">
-        <v>-14.01997037</v>
+        <v>7.23860001</v>
       </c>
       <c r="B67">
-        <v>12.0014248</v>
+        <v>12.74123844</v>
       </c>
       <c r="C67">
-        <v>7.70754394</v>
+        <v>-13.61115399</v>
       </c>
     </row>
     <row r="68">
       <c r="A68">
-        <v>-15.49629546</v>
+        <v>3.87925963</v>
       </c>
       <c r="B68">
-        <v>12.0014248</v>
+        <v>12.6312572</v>
       </c>
       <c r="C68">
-        <v>3.97877242</v>
+        <v>15.01341687</v>
       </c>
     </row>
     <row r="69">
       <c r="A69">
-        <v>-15.9989313</v>
+        <v>-13.07643971</v>
       </c>
       <c r="B69">
-        <v>12.0014248</v>
+        <v>12.52127596</v>
       </c>
       <c r="C69">
-        <v>0</v>
+        <v>-8.49849237</v>
       </c>
     </row>
     <row r="70">
       <c r="A70">
-        <v>-15.49629546</v>
+        <v>15.46928115</v>
       </c>
       <c r="B70">
-        <v>12.0014248</v>
+        <v>12.41129473</v>
       </c>
       <c r="C70">
-        <v>-3.97877242</v>
+        <v>-2.58091146</v>
       </c>
     </row>
     <row r="71">
       <c r="A71">
-        <v>-14.01997037</v>
+        <v>-9.71642959</v>
       </c>
       <c r="B71">
-        <v>12.0014248</v>
+        <v>12.30131349</v>
       </c>
       <c r="C71">
-        <v>-7.70754394</v>
+        <v>12.42049445</v>
       </c>
     </row>
     <row r="72">
       <c r="A72">
-        <v>-11.66271899</v>
+        <v>-1.23194932</v>
       </c>
       <c r="B72">
-        <v>12.0014248</v>
+        <v>12.19133226</v>
       </c>
       <c r="C72">
-        <v>-10.95202212</v>
+        <v>-15.8067618</v>
       </c>
     </row>
     <row r="73">
       <c r="A73">
-        <v>-8.57265608</v>
+        <v>11.64707237</v>
       </c>
       <c r="B73">
-        <v>12.0014248</v>
+        <v>12.08135102</v>
       </c>
       <c r="C73">
-        <v>-13.50834448</v>
+        <v>10.88056353</v>
       </c>
     </row>
     <row r="74">
       <c r="A74">
-        <v>-4.94394166</v>
+        <v>-16.02067015</v>
       </c>
       <c r="B74">
-        <v>12.0014248</v>
+        <v>11.97136979</v>
       </c>
       <c r="C74">
-        <v>-15.21588787</v>
+        <v>-0.15631212</v>
       </c>
     </row>
     <row r="75">
       <c r="A75">
-        <v>-1.00458121</v>
+        <v>11.97943048</v>
       </c>
       <c r="B75">
-        <v>12.0014248</v>
+        <v>11.86138855</v>
       </c>
       <c r="C75">
-        <v>-15.96736107</v>
+        <v>-10.76107369</v>
       </c>
     </row>
     <row r="76">
       <c r="A76">
-        <v>2.99790078</v>
+        <v>-1.57207189</v>
       </c>
       <c r="B76">
-        <v>12.0014248</v>
+        <v>11.75140731</v>
       </c>
       <c r="C76">
-        <v>-15.71554624</v>
+        <v>16.10692448</v>
       </c>
     </row>
     <row r="77">
       <c r="A77">
-        <v>6.81201364</v>
+        <v>-9.76850325</v>
       </c>
       <c r="B77">
-        <v>12.0014248</v>
+        <v>11.64142608</v>
       </c>
       <c r="C77">
-        <v>-14.47626585</v>
+        <v>-13.00205919</v>
       </c>
     </row>
     <row r="78">
       <c r="A78">
-        <v>10.19810262</v>
+        <v>16.06259215</v>
       </c>
       <c r="B78">
-        <v>12.0014248</v>
+        <v>11.53144484</v>
       </c>
       <c r="C78">
-        <v>-12.32738844</v>
+        <v>3.00315054</v>
       </c>
     </row>
     <row r="79">
       <c r="A79">
-        <v>12.94340732</v>
+        <v>-13.9380745</v>
       </c>
       <c r="B79">
-        <v>12.0014248</v>
+        <v>11.42146361</v>
       </c>
       <c r="C79">
-        <v>-9.40393587</v>
+        <v>8.67641909</v>
       </c>
     </row>
     <row r="80">
       <c r="A80">
-        <v>14.87543012</v>
+        <v>4.43710146</v>
       </c>
       <c r="B80">
-        <v>12.0014248</v>
+        <v>11.31148237</v>
       </c>
       <c r="C80">
-        <v>-5.88959943</v>
+        <v>-15.88592135</v>
       </c>
     </row>
     <row r="81">
       <c r="A81">
-        <v>15.87277495</v>
+        <v>7.49287152</v>
       </c>
       <c r="B81">
-        <v>12.0014248</v>
+        <v>11.20150113</v>
       </c>
       <c r="C81">
-        <v>-2.00519779</v>
+        <v>14.7777958</v>
       </c>
     </row>
     <row r="82">
       <c r="A82">
-        <v>17.93745483</v>
+        <v>-15.57636221</v>
       </c>
       <c r="B82">
-        <v>8.8457738</v>
+        <v>11.0915199</v>
       </c>
       <c r="C82">
-        <v>0</v>
+        <v>-5.86132465</v>
       </c>
     </row>
     <row r="83">
       <c r="A83">
-        <v>17.48772539</v>
+        <v>15.51232923</v>
       </c>
       <c r="B83">
-        <v>8.8457738</v>
+        <v>10.98153866</v>
       </c>
       <c r="C83">
-        <v>3.9914592</v>
+        <v>-6.2268331</v>
       </c>
     </row>
     <row r="84">
       <c r="A84">
-        <v>16.16108837</v>
+        <v>-7.26318208</v>
       </c>
       <c r="B84">
-        <v>8.8457738</v>
+        <v>10.87155743</v>
       </c>
       <c r="C84">
-        <v>7.78276997</v>
+        <v>15.13457714</v>
       </c>
     </row>
     <row r="85">
       <c r="A85">
-        <v>14.0240669</v>
+        <v>-4.88812033</v>
       </c>
       <c r="B85">
-        <v>8.8457738</v>
+        <v>10.76157619</v>
       </c>
       <c r="C85">
-        <v>11.18382016</v>
+        <v>-16.13365295</v>
       </c>
     </row>
     <row r="86">
       <c r="A86">
-        <v>11.18382016</v>
+        <v>14.56244022</v>
       </c>
       <c r="B86">
-        <v>8.8457738</v>
+        <v>10.65159496</v>
       </c>
       <c r="C86">
-        <v>14.0240669</v>
+        <v>8.63011354</v>
       </c>
     </row>
     <row r="87">
       <c r="A87">
-        <v>7.78276997</v>
+        <v>-16.63469467</v>
       </c>
       <c r="B87">
-        <v>8.8457738</v>
+        <v>10.54161372</v>
       </c>
       <c r="C87">
-        <v>16.16108837</v>
+        <v>3.48730749</v>
       </c>
     </row>
     <row r="88">
       <c r="A88">
-        <v>3.9914592</v>
+        <v>9.94975186</v>
       </c>
       <c r="B88">
-        <v>8.8457738</v>
+        <v>10.43163248</v>
       </c>
       <c r="C88">
-        <v>17.48772539</v>
+        <v>-13.8630257</v>
       </c>
     </row>
     <row r="89">
       <c r="A89">
-        <v>0</v>
+        <v>2.03563367</v>
       </c>
       <c r="B89">
-        <v>8.8457738</v>
+        <v>10.32165125</v>
       </c>
       <c r="C89">
-        <v>17.93745483</v>
+        <v>17.00940067</v>
       </c>
     </row>
     <row r="90">
       <c r="A90">
-        <v>-3.9914592</v>
+        <v>-13.04058563</v>
       </c>
       <c r="B90">
-        <v>8.8457738</v>
+        <v>10.21167001</v>
       </c>
       <c r="C90">
-        <v>17.48772539</v>
+        <v>-11.21003666</v>
       </c>
     </row>
     <row r="91">
       <c r="A91">
-        <v>-7.78276997</v>
+        <v>17.25279583</v>
       </c>
       <c r="B91">
-        <v>8.8457738</v>
+        <v>10.10168878</v>
       </c>
       <c r="C91">
-        <v>16.16108837</v>
+        <v>-0.54490357</v>
       </c>
     </row>
     <row r="92">
       <c r="A92">
-        <v>-11.18382016</v>
+        <v>-12.39932544</v>
       </c>
       <c r="B92">
-        <v>8.8457738</v>
+        <v>9.99170754</v>
       </c>
       <c r="C92">
-        <v>14.0240669</v>
+        <v>12.10051689</v>
       </c>
     </row>
     <row r="93">
       <c r="A93">
-        <v>-14.0240669</v>
+        <v>0.97261689</v>
       </c>
       <c r="B93">
-        <v>8.8457738</v>
+        <v>9.88172631</v>
       </c>
       <c r="C93">
-        <v>11.18382016</v>
+        <v>-17.361034</v>
       </c>
     </row>
     <row r="94">
       <c r="A94">
-        <v>-16.16108837</v>
+        <v>11.04931786</v>
       </c>
       <c r="B94">
-        <v>8.8457738</v>
+        <v>9.77174507</v>
       </c>
       <c r="C94">
-        <v>7.78276997</v>
+        <v>13.50650114</v>
       </c>
     </row>
     <row r="95">
       <c r="A95">
-        <v>-17.48772539</v>
+        <v>-17.33143833</v>
       </c>
       <c r="B95">
-        <v>8.8457738</v>
+        <v>9.66176383</v>
       </c>
       <c r="C95">
-        <v>3.9914592</v>
+        <v>-2.50430927</v>
       </c>
     </row>
     <row r="96">
       <c r="A96">
-        <v>-17.93745483</v>
+        <v>14.52107516</v>
       </c>
       <c r="B96">
-        <v>8.8457738</v>
+        <v>9.5517826</v>
       </c>
       <c r="C96">
-        <v>0</v>
+        <v>-9.89453513</v>
       </c>
     </row>
     <row r="97">
       <c r="A97">
-        <v>-17.48772539</v>
+        <v>-4.03731476</v>
       </c>
       <c r="B97">
-        <v>8.8457738</v>
+        <v>9.44180136</v>
       </c>
       <c r="C97">
-        <v>-3.9914592</v>
+        <v>17.16253118</v>
       </c>
     </row>
     <row r="98">
       <c r="A98">
-        <v>-16.16108837</v>
+        <v>-8.6447007</v>
       </c>
       <c r="B98">
-        <v>8.8457738</v>
+        <v>9.33182013</v>
       </c>
       <c r="C98">
-        <v>-7.78276997</v>
+        <v>-15.43328491</v>
       </c>
     </row>
     <row r="99">
       <c r="A99">
-        <v>-14.0240669</v>
+        <v>16.85405333</v>
       </c>
       <c r="B99">
-        <v>8.8457738</v>
+        <v>9.22183889</v>
       </c>
       <c r="C99">
-        <v>-11.18382016</v>
+        <v>5.55864856</v>
       </c>
     </row>
     <row r="100">
       <c r="A100">
-        <v>-11.18382016</v>
+        <v>-16.23418507</v>
       </c>
       <c r="B100">
-        <v>8.8457738</v>
+        <v>9.11185765</v>
       </c>
       <c r="C100">
-        <v>-14.0240669</v>
+        <v>7.30926023</v>
       </c>
     </row>
     <row r="101">
       <c r="A101">
-        <v>-7.78276997</v>
+        <v>7.05531574</v>
       </c>
       <c r="B101">
-        <v>8.8457738</v>
+        <v>9.00187642</v>
       </c>
       <c r="C101">
-        <v>-16.16108837</v>
+        <v>-16.40697232</v>
       </c>
     </row>
     <row r="102">
       <c r="A102">
-        <v>-3.9914592</v>
+        <v>5.898493</v>
       </c>
       <c r="B102">
-        <v>8.8457738</v>
+        <v>8.89189518</v>
       </c>
       <c r="C102">
-        <v>-17.48772539</v>
+        <v>16.91573174</v>
       </c>
     </row>
     <row r="103">
       <c r="A103">
-        <v>0</v>
+        <v>-15.82347987</v>
       </c>
       <c r="B103">
-        <v>8.8457738</v>
+        <v>8.78191395</v>
       </c>
       <c r="C103">
-        <v>-17.93745483</v>
+        <v>-8.5144273</v>
       </c>
     </row>
     <row r="104">
       <c r="A104">
-        <v>3.9914592</v>
+        <v>17.47085862</v>
       </c>
       <c r="B104">
-        <v>8.8457738</v>
+        <v>8.67193271</v>
       </c>
       <c r="C104">
-        <v>-17.48772539</v>
+        <v>-4.42342425</v>
       </c>
     </row>
     <row r="105">
       <c r="A105">
-        <v>7.78276997</v>
+        <v>-9.92331564</v>
       </c>
       <c r="B105">
-        <v>8.8457738</v>
+        <v>8.56195148</v>
       </c>
       <c r="C105">
-        <v>-16.16108837</v>
+        <v>15.10697831</v>
       </c>
     </row>
     <row r="106">
       <c r="A106">
-        <v>11.18382016</v>
+        <v>-2.89573064</v>
       </c>
       <c r="B106">
-        <v>8.8457738</v>
+        <v>8.45197024</v>
       </c>
       <c r="C106">
-        <v>-14.0240669</v>
+        <v>-17.89354473</v>
       </c>
     </row>
     <row r="107">
       <c r="A107">
-        <v>14.0240669</v>
+        <v>14.26205623</v>
       </c>
       <c r="B107">
-        <v>8.8457738</v>
+        <v>8.341989</v>
       </c>
       <c r="C107">
-        <v>-11.18382016</v>
+        <v>11.26964825</v>
       </c>
     </row>
     <row r="108">
       <c r="A108">
-        <v>16.16108837</v>
+        <v>-18.17887292</v>
       </c>
       <c r="B108">
-        <v>8.8457738</v>
+        <v>8.23200777</v>
       </c>
       <c r="C108">
-        <v>-7.78276997</v>
+        <v>1.32763979</v>
       </c>
     </row>
     <row r="109">
       <c r="A109">
-        <v>17.48772539</v>
+        <v>12.54153859</v>
       </c>
       <c r="B109">
-        <v>8.8457738</v>
+        <v>8.12202653</v>
       </c>
       <c r="C109">
-        <v>-3.9914592</v>
+        <v>-13.29445354</v>
       </c>
     </row>
     <row r="110">
       <c r="A110">
-        <v>19.15538949</v>
+        <v>-0.26817538</v>
       </c>
       <c r="B110">
-        <v>5.38680108</v>
+        <v>8.0120453</v>
       </c>
       <c r="C110">
-        <v>2.01331256</v>
+        <v>18.32307868</v>
       </c>
     </row>
     <row r="111">
       <c r="A111">
-        <v>18.31820706</v>
+        <v>-12.21101616</v>
       </c>
       <c r="B111">
-        <v>5.38680108</v>
+        <v>7.90206406</v>
       </c>
       <c r="C111">
-        <v>5.95194627</v>
+        <v>-13.7276534</v>
       </c>
     </row>
     <row r="112">
       <c r="A112">
-        <v>16.68043107</v>
+        <v>18.32358883</v>
       </c>
       <c r="B112">
-        <v>5.38680108</v>
+        <v>7.79208282</v>
       </c>
       <c r="C112">
-        <v>9.63045137</v>
+        <v>1.87870642</v>
       </c>
     </row>
     <row r="113">
       <c r="A113">
-        <v>14.3136402</v>
+        <v>-14.81731522</v>
       </c>
       <c r="B113">
-        <v>5.38680108</v>
+        <v>7.68210159</v>
       </c>
       <c r="C113">
-        <v>12.88805953</v>
+        <v>11.01964087</v>
       </c>
     </row>
     <row r="114">
       <c r="A114">
-        <v>11.32127457</v>
+        <v>3.49072241</v>
       </c>
       <c r="B114">
-        <v>5.38680108</v>
+        <v>7.57212035</v>
       </c>
       <c r="C114">
-        <v>15.58239764</v>
+        <v>-18.17904977</v>
       </c>
     </row>
     <row r="115">
       <c r="A115">
-        <v>7.83411492</v>
+        <v>9.72921067</v>
       </c>
       <c r="B115">
-        <v>5.38680108</v>
+        <v>7.46213912</v>
       </c>
       <c r="C115">
-        <v>17.5957102</v>
+        <v>15.80059934</v>
       </c>
     </row>
     <row r="116">
       <c r="A116">
-        <v>4.00456685</v>
+        <v>-17.88934494</v>
       </c>
       <c r="B116">
-        <v>5.38680108</v>
+        <v>7.35215788</v>
       </c>
       <c r="C116">
-        <v>18.8400058</v>
+        <v>-5.09088521</v>
       </c>
     </row>
     <row r="117">
       <c r="A117">
-        <v>0</v>
+        <v>16.6684244</v>
       </c>
       <c r="B117">
-        <v>5.38680108</v>
+        <v>7.24217665</v>
       </c>
       <c r="C117">
-        <v>19.26090273</v>
+        <v>-8.34952127</v>
       </c>
     </row>
     <row r="118">
       <c r="A118">
-        <v>-4.00456685</v>
+        <v>-6.66586587</v>
       </c>
       <c r="B118">
-        <v>5.38680108</v>
+        <v>7.13219541</v>
       </c>
       <c r="C118">
-        <v>18.8400058</v>
+        <v>17.45560142</v>
       </c>
     </row>
     <row r="119">
       <c r="A119">
-        <v>-7.83411492</v>
+        <v>-6.89119946</v>
       </c>
       <c r="B119">
-        <v>5.38680108</v>
+        <v>7.02221417</v>
       </c>
       <c r="C119">
-        <v>17.5957102</v>
+        <v>-17.41263559</v>
       </c>
     </row>
     <row r="120">
       <c r="A120">
-        <v>-11.32127457</v>
+        <v>16.88018556</v>
       </c>
       <c r="B120">
-        <v>5.38680108</v>
+        <v>6.91223294</v>
       </c>
       <c r="C120">
-        <v>15.58239764</v>
+        <v>8.20246128</v>
       </c>
     </row>
     <row r="121">
       <c r="A121">
-        <v>-14.3136402</v>
+        <v>-18.02608</v>
       </c>
       <c r="B121">
-        <v>5.38680108</v>
+        <v>6.8022517</v>
       </c>
       <c r="C121">
-        <v>12.88805953</v>
+        <v>5.36561381</v>
       </c>
     </row>
     <row r="122">
       <c r="A122">
-        <v>-16.68043107</v>
+        <v>9.68771</v>
       </c>
       <c r="B122">
-        <v>5.38680108</v>
+        <v>6.69227047</v>
       </c>
       <c r="C122">
-        <v>9.63045137</v>
+        <v>-16.1666877</v>
       </c>
     </row>
     <row r="123">
       <c r="A123">
-        <v>-18.31820706</v>
+        <v>3.78477874</v>
       </c>
       <c r="B123">
-        <v>5.38680108</v>
+        <v>6.58228923</v>
       </c>
       <c r="C123">
-        <v>5.95194627</v>
+        <v>18.50267328</v>
       </c>
     </row>
     <row r="124">
       <c r="A124">
-        <v>-19.15538949</v>
+        <v>-15.319896</v>
       </c>
       <c r="B124">
-        <v>5.38680108</v>
+        <v>6.47230799</v>
       </c>
       <c r="C124">
-        <v>2.01331256</v>
+        <v>-11.10900607</v>
       </c>
     </row>
     <row r="125">
       <c r="A125">
-        <v>-19.15538949</v>
+        <v>18.83745697</v>
       </c>
       <c r="B125">
-        <v>5.38680108</v>
+        <v>6.36232676</v>
       </c>
       <c r="C125">
-        <v>-2.01331256</v>
+        <v>-2.1612527</v>
       </c>
     </row>
     <row r="126">
       <c r="A126">
-        <v>-18.31820706</v>
+        <v>-12.45421013</v>
       </c>
       <c r="B126">
-        <v>5.38680108</v>
+        <v>6.25234552</v>
       </c>
       <c r="C126">
-        <v>-5.95194627</v>
+        <v>14.34575985</v>
       </c>
     </row>
     <row r="127">
       <c r="A127">
-        <v>-16.68043107</v>
+        <v>-0.50803133</v>
       </c>
       <c r="B127">
-        <v>5.38680108</v>
+        <v>6.14236429</v>
       </c>
       <c r="C127">
-        <v>-9.63045137</v>
+        <v>-19.02664619</v>
       </c>
     </row>
     <row r="128">
       <c r="A128">
-        <v>-14.3136402</v>
+        <v>13.25134283</v>
       </c>
       <c r="B128">
-        <v>5.38680108</v>
+        <v>6.03238305</v>
       </c>
       <c r="C128">
-        <v>-12.88805953</v>
+        <v>13.71175655</v>
       </c>
     </row>
     <row r="129">
       <c r="A129">
-        <v>-11.32127457</v>
+        <v>-19.06766706</v>
       </c>
       <c r="B129">
-        <v>5.38680108</v>
+        <v>5.92240182</v>
       </c>
       <c r="C129">
-        <v>-15.58239764</v>
+        <v>-1.16156348</v>
       </c>
     </row>
     <row r="130">
       <c r="A130">
-        <v>-7.83411492</v>
+        <v>14.87075586</v>
       </c>
       <c r="B130">
-        <v>5.38680108</v>
+        <v>5.81242058</v>
       </c>
       <c r="C130">
-        <v>-17.5957102</v>
+        <v>-12.04476596</v>
       </c>
     </row>
     <row r="131">
       <c r="A131">
-        <v>-4.00456685</v>
+        <v>-2.83399754</v>
       </c>
       <c r="B131">
-        <v>5.38680108</v>
+        <v>5.70243934</v>
       </c>
       <c r="C131">
-        <v>-18.8400058</v>
+        <v>18.95918362</v>
       </c>
     </row>
     <row r="132">
       <c r="A132">
-        <v>0</v>
+        <v>-10.73514145</v>
       </c>
       <c r="B132">
-        <v>5.38680108</v>
+        <v>5.59245811</v>
       </c>
       <c r="C132">
-        <v>-19.26090273</v>
+        <v>-15.92109137</v>
       </c>
     </row>
     <row r="133">
       <c r="A133">
-        <v>4.00456685</v>
+        <v>18.70111398</v>
       </c>
       <c r="B133">
-        <v>5.38680108</v>
+        <v>5.48247687</v>
       </c>
       <c r="C133">
-        <v>-18.8400058</v>
+        <v>4.49564047</v>
       </c>
     </row>
     <row r="134">
       <c r="A134">
-        <v>7.83411492</v>
+        <v>-16.85350932</v>
       </c>
       <c r="B134">
-        <v>5.38680108</v>
+        <v>5.37249564</v>
       </c>
       <c r="C134">
-        <v>-17.5957102</v>
+        <v>9.33249774</v>
       </c>
     </row>
     <row r="135">
       <c r="A135">
-        <v>11.32127457</v>
+        <v>6.13288285</v>
       </c>
       <c r="B135">
-        <v>5.38680108</v>
+        <v>5.2625144</v>
       </c>
       <c r="C135">
-        <v>-15.58239764</v>
+        <v>-18.29463556</v>
       </c>
     </row>
     <row r="136">
       <c r="A136">
-        <v>14.3136402</v>
+        <v>7.84769638</v>
       </c>
       <c r="B136">
-        <v>5.38680108</v>
+        <v>5.15253317</v>
       </c>
       <c r="C136">
-        <v>-12.88805953</v>
+        <v>17.65970168</v>
       </c>
     </row>
     <row r="137">
       <c r="A137">
-        <v>16.68043107</v>
+        <v>-17.74217931</v>
       </c>
       <c r="B137">
-        <v>5.38680108</v>
+        <v>5.04255193</v>
       </c>
       <c r="C137">
-        <v>-9.63045137</v>
+        <v>-7.73225345</v>
       </c>
     </row>
     <row r="138">
       <c r="A138">
-        <v>18.31820706</v>
+        <v>18.3323808</v>
       </c>
       <c r="B138">
-        <v>5.38680108</v>
+        <v>4.93257069</v>
       </c>
       <c r="C138">
-        <v>-5.95194627</v>
+        <v>-6.29234142</v>
       </c>
     </row>
     <row r="139">
       <c r="A139">
-        <v>19.15538949</v>
+        <v>-9.28053544</v>
       </c>
       <c r="B139">
-        <v>5.38680108</v>
+        <v>4.82258946</v>
       </c>
       <c r="C139">
-        <v>-2.01331256</v>
+        <v>17.04741308</v>
       </c>
     </row>
     <row r="140">
       <c r="A140">
-        <v>19.92389396</v>
+        <v>-4.67868225</v>
       </c>
       <c r="B140">
-        <v>1.74311485</v>
+        <v>4.71260822</v>
       </c>
       <c r="C140">
-        <v>0</v>
+        <v>-18.86534538</v>
       </c>
     </row>
     <row r="141">
       <c r="A141">
-        <v>19.51605068</v>
+        <v>16.21521411</v>
       </c>
       <c r="B141">
-        <v>1.74311485</v>
+        <v>4.60262699</v>
       </c>
       <c r="C141">
-        <v>4.01065037</v>
+        <v>10.76488068</v>
       </c>
     </row>
     <row r="142">
       <c r="A142">
-        <v>18.30921799</v>
+        <v>-19.25353708</v>
       </c>
       <c r="B142">
-        <v>1.74311485</v>
+        <v>4.49264575</v>
       </c>
       <c r="C142">
-        <v>7.85710424</v>
+        <v>3.01951058</v>
       </c>
     </row>
     <row r="143">
       <c r="A143">
-        <v>16.35280377</v>
+        <v>12.1729209</v>
       </c>
       <c r="B143">
-        <v>1.74311485</v>
+        <v>4.38266451</v>
       </c>
       <c r="C143">
-        <v>11.38188734</v>
+        <v>-15.25163101</v>
       </c>
     </row>
     <row r="144">
       <c r="A144">
-        <v>13.72690384</v>
+        <v>1.32805255</v>
       </c>
       <c r="B144">
-        <v>1.74311485</v>
+        <v>4.27268328</v>
       </c>
       <c r="C144">
-        <v>14.44069464</v>
+        <v>19.49308734</v>
       </c>
     </row>
     <row r="145">
       <c r="A145">
-        <v>10.53902285</v>
+        <v>-14.16383545</v>
       </c>
       <c r="B145">
-        <v>1.74311485</v>
+        <v>4.16270204</v>
       </c>
       <c r="C145">
-        <v>16.9082982</v>
+        <v>-13.49287504</v>
       </c>
     </row>
     <row r="146">
       <c r="A146">
-        <v>6.91967303</v>
+        <v>19.5813539</v>
       </c>
       <c r="B146">
-        <v>1.74311485</v>
+        <v>4.05272081</v>
       </c>
       <c r="C146">
-        <v>18.68367404</v>
+        <v>0.38214311</v>
       </c>
     </row>
     <row r="147">
       <c r="A147">
-        <v>3.01703098</v>
+        <v>-14.71365157</v>
       </c>
       <c r="B147">
-        <v>1.74311485</v>
+        <v>3.94273957</v>
       </c>
       <c r="C147">
-        <v>19.69413808</v>
+        <v>12.96006412</v>
       </c>
     </row>
     <row r="148">
       <c r="A148">
-        <v>-1.00912867</v>
+        <v>2.09731992</v>
       </c>
       <c r="B148">
-        <v>1.74311485</v>
+        <v>3.83275834</v>
       </c>
       <c r="C148">
-        <v>19.89832179</v>
+        <v>-19.51694681</v>
       </c>
     </row>
     <row r="149">
       <c r="A149">
-        <v>-4.99397447</v>
+        <v>11.64955125</v>
       </c>
       <c r="B149">
-        <v>1.74311485</v>
+        <v>3.7227771</v>
       </c>
       <c r="C149">
-        <v>19.28786586</v>
+        <v>15.82494506</v>
       </c>
     </row>
     <row r="150">
       <c r="A150">
-        <v>-8.77436638</v>
+        <v>-19.29974355</v>
       </c>
       <c r="B150">
-        <v>1.74311485</v>
+        <v>3.61279586</v>
       </c>
       <c r="C150">
-        <v>17.88776244</v>
+        <v>-3.80363049</v>
       </c>
     </row>
     <row r="151">
       <c r="A151">
-        <v>-12.19553469</v>
+        <v>16.8173261</v>
       </c>
       <c r="B151">
-        <v>1.74311485</v>
+        <v>3.50281463</v>
       </c>
       <c r="C151">
-        <v>15.75533193</v>
+        <v>-10.24245246</v>
       </c>
     </row>
     <row r="152">
       <c r="A152">
-        <v>-15.11741638</v>
+        <v>-5.48725427</v>
       </c>
       <c r="B152">
-        <v>1.74311485</v>
+        <v>3.39283339</v>
       </c>
       <c r="C152">
-        <v>12.97787628</v>
+        <v>18.93089333</v>
       </c>
     </row>
     <row r="153">
       <c r="A153">
-        <v>-17.42038927</v>
+        <v>-8.74976052</v>
       </c>
       <c r="B153">
-        <v>1.74311485</v>
+        <v>3.28285216</v>
       </c>
       <c r="C153">
-        <v>9.66910484</v>
+        <v>-17.68232373</v>
       </c>
     </row>
     <row r="154">
       <c r="A154">
-        <v>-19.01016937</v>
+        <v>18.41281026</v>
       </c>
       <c r="B154">
-        <v>1.74311485</v>
+        <v>3.17287092</v>
       </c>
       <c r="C154">
-        <v>5.96447912</v>
+        <v>7.1345153</v>
       </c>
     </row>
     <row r="155">
       <c r="A155">
-        <v>-19.82167091</v>
+        <v>-18.41249977</v>
       </c>
       <c r="B155">
-        <v>1.74311485</v>
+        <v>3.06288968</v>
       </c>
       <c r="C155">
-        <v>2.01566692</v>
+        <v>7.1832137</v>
       </c>
     </row>
     <row r="156">
       <c r="A156">
-        <v>-19.82167091</v>
+        <v>8.73199885</v>
       </c>
       <c r="B156">
-        <v>1.74311485</v>
+        <v>2.95290845</v>
       </c>
       <c r="C156">
-        <v>-2.01566692</v>
+        <v>-17.74915569</v>
       </c>
     </row>
     <row r="157">
       <c r="A157">
-        <v>-19.01016937</v>
+        <v>5.55519765</v>
       </c>
       <c r="B157">
-        <v>1.74311485</v>
+        <v>2.84292721</v>
       </c>
       <c r="C157">
-        <v>-5.96447912</v>
+        <v>19.00151425</v>
       </c>
     </row>
     <row r="158">
       <c r="A158">
-        <v>-17.42038927</v>
+        <v>-16.94480972</v>
       </c>
       <c r="B158">
-        <v>1.74311485</v>
+        <v>2.73294598</v>
       </c>
       <c r="C158">
-        <v>-9.66910484</v>
+        <v>-10.26666596</v>
       </c>
     </row>
     <row r="159">
       <c r="A159">
-        <v>-15.11741638</v>
+        <v>19.44418155</v>
       </c>
       <c r="B159">
-        <v>1.74311485</v>
+        <v>2.62296474</v>
       </c>
       <c r="C159">
-        <v>-12.97787628</v>
+        <v>-3.8786415</v>
       </c>
     </row>
     <row r="160">
       <c r="A160">
-        <v>-12.19553469</v>
+        <v>-11.72596485</v>
       </c>
       <c r="B160">
-        <v>1.74311485</v>
+        <v>2.51298351</v>
       </c>
       <c r="C160">
-        <v>-15.75533193</v>
+        <v>16.00583213</v>
       </c>
     </row>
     <row r="161">
       <c r="A161">
-        <v>-8.77436638</v>
+        <v>-2.16690914</v>
       </c>
       <c r="B161">
-        <v>1.74311485</v>
+        <v>2.40300227</v>
       </c>
       <c r="C161">
-        <v>-17.88776244</v>
+        <v>-19.73651653</v>
       </c>
     </row>
     <row r="162">
       <c r="A162">
-        <v>-4.99397447</v>
+        <v>14.93941317</v>
       </c>
       <c r="B162">
-        <v>1.74311485</v>
+        <v>2.29302103</v>
       </c>
       <c r="C162">
-        <v>-19.28786586</v>
+        <v>13.09793834</v>
       </c>
     </row>
     <row r="163">
       <c r="A163">
-        <v>-1.00912867</v>
+        <v>-19.8757705</v>
       </c>
       <c r="B163">
-        <v>1.74311485</v>
+        <v>2.1830398</v>
       </c>
       <c r="C163">
-        <v>-19.89832179</v>
+        <v>0.43368667</v>
       </c>
     </row>
     <row r="164">
       <c r="A164">
-        <v>3.01703098</v>
+        <v>14.37132616</v>
       </c>
       <c r="B164">
-        <v>1.74311485</v>
+        <v>2.07305856</v>
       </c>
       <c r="C164">
-        <v>-19.69413808</v>
+        <v>-13.75381447</v>
       </c>
     </row>
     <row r="165">
       <c r="A165">
-        <v>6.91967303</v>
+        <v>-1.30713302</v>
       </c>
       <c r="B165">
-        <v>1.74311485</v>
+        <v>1.96307733</v>
       </c>
       <c r="C165">
-        <v>-18.68367404</v>
+        <v>19.86045646</v>
       </c>
     </row>
     <row r="166">
       <c r="A166">
-        <v>10.53902285</v>
+        <v>-12.45830077</v>
       </c>
       <c r="B166">
-        <v>1.74311485</v>
+        <v>1.85309609</v>
       </c>
       <c r="C166">
-        <v>-16.9082982</v>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167">
-        <v>13.72690384</v>
-      </c>
-      <c r="B167">
-        <v>1.74311485</v>
-      </c>
-      <c r="C167">
-        <v>-14.44069464</v>
-      </c>
-    </row>
-    <row r="168">
-      <c r="A168">
-        <v>16.35280377</v>
-      </c>
-      <c r="B168">
-        <v>1.74311485</v>
-      </c>
-      <c r="C168">
-        <v>-11.38188734</v>
-      </c>
-    </row>
-    <row r="169">
-      <c r="A169">
-        <v>18.30921799</v>
-      </c>
-      <c r="B169">
-        <v>1.74311485</v>
-      </c>
-      <c r="C169">
-        <v>-7.85710424</v>
-      </c>
-    </row>
-    <row r="170">
-      <c r="A170">
-        <v>19.51605068</v>
-      </c>
-      <c r="B170">
-        <v>1.74311485</v>
-      </c>
-      <c r="C170">
-        <v>-4.01065037</v>
+        <v>-15.53566146</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
towards more symmetric pin placement when using Fibonacci
</commit_message>
<xml_diff>
--- a/pin_points_inventor.xlsx
+++ b/pin_points_inventor.xlsx
@@ -23,10 +23,10 @@
     </row>
     <row r="2">
       <c r="A2">
-        <v>2.09455331</v>
+        <v>3.97338662</v>
       </c>
       <c r="B2">
-        <v>19.89001876</v>
+        <v>19.60133156</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -34,1806 +34,1806 @@
     </row>
     <row r="3">
       <c r="A3">
-        <v>-2.18118094</v>
+        <v>1.98669331</v>
       </c>
       <c r="B3">
-        <v>19.78003753</v>
+        <v>19.60133156</v>
       </c>
       <c r="C3">
-        <v>1.99814041</v>
+        <v>3.44105375</v>
       </c>
     </row>
     <row r="4">
       <c r="A4">
-        <v>0.31629372</v>
+        <v>-1.98669331</v>
       </c>
       <c r="B4">
-        <v>19.67005629</v>
+        <v>19.60133156</v>
       </c>
       <c r="C4">
-        <v>-3.60400385</v>
+        <v>3.44105375</v>
       </c>
     </row>
     <row r="5">
       <c r="A5">
-        <v>2.53825232</v>
+        <v>-3.97338662</v>
       </c>
       <c r="B5">
-        <v>19.56007506</v>
+        <v>19.60133156</v>
       </c>
       <c r="C5">
-        <v>3.31070067</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6">
-        <v>-4.58646629</v>
+        <v>-1.98669331</v>
       </c>
       <c r="B6">
-        <v>19.45009382</v>
+        <v>19.60133156</v>
       </c>
       <c r="C6">
-        <v>-0.81128131</v>
+        <v>-3.44105375</v>
       </c>
     </row>
     <row r="7">
       <c r="A7">
-        <v>4.2990177</v>
+        <v>1.98669331</v>
       </c>
       <c r="B7">
-        <v>19.34011259</v>
+        <v>19.60133156</v>
       </c>
       <c r="C7">
-        <v>-2.73468316</v>
+        <v>-3.44105375</v>
       </c>
     </row>
     <row r="8">
       <c r="A8">
-        <v>-1.42669155</v>
+        <v>2.05632353</v>
       </c>
       <c r="B8">
-        <v>19.23013135</v>
+        <v>19.1780916</v>
       </c>
       <c r="C8">
-        <v>5.30722145</v>
+        <v>5.28888798</v>
       </c>
     </row>
     <row r="9">
       <c r="A9">
-        <v>-2.70406966</v>
+        <v>-5.41109251</v>
       </c>
       <c r="B9">
-        <v>19.12015011</v>
+        <v>19.06809175</v>
       </c>
       <c r="C9">
-        <v>-5.20652158</v>
+        <v>-2.66982301</v>
       </c>
     </row>
     <row r="10">
       <c r="A10">
-        <v>5.83691859</v>
+        <v>6.11716492</v>
       </c>
       <c r="B10">
-        <v>19.01016888</v>
+        <v>18.9580919</v>
       </c>
       <c r="C10">
-        <v>2.13163331</v>
+        <v>-1.78074283</v>
       </c>
     </row>
     <row r="11">
       <c r="A11">
-        <v>-6.04601894</v>
+        <v>-3.47304631</v>
       </c>
       <c r="B11">
-        <v>18.90018764</v>
+        <v>18.84809204</v>
       </c>
       <c r="C11">
-        <v>2.49570873</v>
+        <v>5.71728744</v>
       </c>
     </row>
     <row r="12">
       <c r="A12">
-        <v>2.90351965</v>
+        <v>-1.35983167</v>
       </c>
       <c r="B12">
-        <v>18.79020641</v>
+        <v>18.73809219</v>
       </c>
       <c r="C12">
-        <v>-6.20465284</v>
+        <v>-6.85818919</v>
       </c>
     </row>
     <row r="13">
       <c r="A13">
-        <v>2.13834473</v>
+        <v>5.86747295</v>
       </c>
       <c r="B13">
-        <v>18.68022517</v>
+        <v>18.62809234</v>
       </c>
       <c r="C13">
-        <v>6.81737995</v>
+        <v>4.30893689</v>
       </c>
     </row>
     <row r="14">
       <c r="A14">
-        <v>-6.42509131</v>
+        <v>-7.51096362</v>
       </c>
       <c r="B14">
-        <v>18.57024393</v>
+        <v>18.51809248</v>
       </c>
       <c r="C14">
-        <v>-3.72347175</v>
+        <v>0.81588991</v>
       </c>
     </row>
     <row r="15">
       <c r="A15">
-        <v>7.51588028</v>
+        <v>5.16162324</v>
       </c>
       <c r="B15">
-        <v>18.4602627</v>
+        <v>18.40809263</v>
       </c>
       <c r="C15">
-        <v>-1.6523452</v>
+        <v>-5.87365059</v>
       </c>
     </row>
     <row r="16">
       <c r="A16">
-        <v>-4.57461759</v>
+        <v>0.1668233</v>
       </c>
       <c r="B16">
-        <v>18.35028146</v>
+        <v>18.29809278</v>
       </c>
       <c r="C16">
-        <v>6.50692278</v>
+        <v>8.07167707</v>
       </c>
     </row>
     <row r="17">
       <c r="A17">
-        <v>-1.05419072</v>
+        <v>-5.74443811</v>
       </c>
       <c r="B17">
-        <v>18.24030023</v>
+        <v>18.18809292</v>
       </c>
       <c r="C17">
-        <v>-8.13511706</v>
+        <v>-6.01620367</v>
       </c>
     </row>
     <row r="18">
       <c r="A18">
-        <v>6.45626131</v>
+        <v>8.53555912</v>
       </c>
       <c r="B18">
-        <v>18.13031899</v>
+        <v>18.07809307</v>
       </c>
       <c r="C18">
-        <v>5.44134387</v>
+        <v>0.57164813</v>
       </c>
     </row>
     <row r="19">
       <c r="A19">
-        <v>-8.66827165</v>
+        <v>-6.85857466</v>
       </c>
       <c r="B19">
-        <v>18.02033776</v>
+        <v>17.96809322</v>
       </c>
       <c r="C19">
-        <v>0.35846025</v>
+        <v>5.48703743</v>
       </c>
     </row>
     <row r="20">
       <c r="A20">
-        <v>6.30894532</v>
+        <v>1.38493173</v>
       </c>
       <c r="B20">
-        <v>17.91035652</v>
+        <v>17.85809336</v>
       </c>
       <c r="C20">
-        <v>-6.27824324</v>
+        <v>-8.89777869</v>
       </c>
     </row>
     <row r="21">
       <c r="A21">
-        <v>-0.42119568</v>
+        <v>5.10822798</v>
       </c>
       <c r="B21">
-        <v>17.80037528</v>
+        <v>17.74809351</v>
       </c>
       <c r="C21">
-        <v>9.10874492</v>
+        <v>7.67536212</v>
       </c>
     </row>
     <row r="22">
       <c r="A22">
-        <v>-5.97785266</v>
+        <v>-9.15393126</v>
       </c>
       <c r="B22">
-        <v>17.69039405</v>
+        <v>17.63809366</v>
       </c>
       <c r="C22">
-        <v>-7.16346536</v>
+        <v>-2.25902517</v>
       </c>
     </row>
     <row r="23">
       <c r="A23">
-        <v>9.45051518</v>
+        <v>8.45391158</v>
       </c>
       <c r="B23">
-        <v>17.58041281</v>
+        <v>17.5280938</v>
       </c>
       <c r="C23">
-        <v>1.27155345</v>
+        <v>-4.61490049</v>
       </c>
     </row>
     <row r="24">
       <c r="A24">
-        <v>-7.99163751</v>
+        <v>-3.18024337</v>
       </c>
       <c r="B24">
-        <v>17.47043158</v>
+        <v>17.41809395</v>
       </c>
       <c r="C24">
-        <v>5.56037323</v>
+        <v>9.30032555</v>
       </c>
     </row>
     <row r="25">
       <c r="A25">
-        <v>2.179559</v>
+        <v>-4.01435065</v>
       </c>
       <c r="B25">
-        <v>17.36045034</v>
+        <v>17.3080941</v>
       </c>
       <c r="C25">
-        <v>-9.6883583</v>
+        <v>-9.18231276</v>
       </c>
     </row>
     <row r="26">
       <c r="A26">
-        <v>5.03164033</v>
+        <v>9.33416195</v>
       </c>
       <c r="B26">
-        <v>17.2504691</v>
+        <v>17.19809424</v>
       </c>
       <c r="C26">
-        <v>8.78088328</v>
+        <v>4.13509071</v>
       </c>
     </row>
     <row r="27">
       <c r="A27">
-        <v>-9.81799138</v>
+        <v>-9.84944375</v>
       </c>
       <c r="B27">
-        <v>17.14048787</v>
+        <v>17.08809439</v>
       </c>
       <c r="C27">
-        <v>-3.13220703</v>
+        <v>3.31443631</v>
       </c>
     </row>
     <row r="28">
       <c r="A28">
-        <v>9.51934229</v>
+        <v>5.11021837</v>
       </c>
       <c r="B28">
-        <v>17.03050663</v>
+        <v>16.97809454</v>
       </c>
       <c r="C28">
-        <v>-4.39817759</v>
+        <v>-9.25364653</v>
       </c>
     </row>
     <row r="29">
       <c r="A29">
-        <v>-4.11650146</v>
+        <v>2.52365151</v>
       </c>
       <c r="B29">
-        <v>16.9205254</v>
+        <v>16.86809468</v>
       </c>
       <c r="C29">
-        <v>9.83616979</v>
+        <v>10.44502584</v>
       </c>
     </row>
     <row r="30">
       <c r="A30">
-        <v>-3.66726133</v>
+        <v>-9.05806325</v>
       </c>
       <c r="B30">
-        <v>16.81054416</v>
+        <v>16.75809483</v>
       </c>
       <c r="C30">
-        <v>-10.19592072</v>
+        <v>-6.09243365</v>
       </c>
     </row>
     <row r="31">
       <c r="A31">
-        <v>9.74075255</v>
+        <v>10.95968286</v>
       </c>
       <c r="B31">
-        <v>16.70056293</v>
+        <v>16.64809498</v>
       </c>
       <c r="C31">
-        <v>5.11946655</v>
+        <v>-1.65114664</v>
       </c>
     </row>
     <row r="32">
       <c r="A32">
-        <v>-10.80034937</v>
+        <v>-7.06874237</v>
       </c>
       <c r="B32">
-        <v>16.59058169</v>
+        <v>16.53809512</v>
       </c>
       <c r="C32">
-        <v>2.84693743</v>
+        <v>8.74781636</v>
       </c>
     </row>
     <row r="33">
       <c r="A33">
-        <v>6.12819059</v>
+        <v>-0.70671175</v>
       </c>
       <c r="B33">
-        <v>16.48060045</v>
+        <v>16.42809527</v>
       </c>
       <c r="C33">
-        <v>-9.5307444</v>
+        <v>-11.38500085</v>
       </c>
     </row>
     <row r="34">
       <c r="A34">
-        <v>1.9460049</v>
+        <v>8.32445017</v>
       </c>
       <c r="B34">
-        <v>16.37061922</v>
+        <v>16.31809542</v>
       </c>
       <c r="C34">
-        <v>11.32324562</v>
+        <v>8.02641211</v>
       </c>
     </row>
     <row r="35">
       <c r="A35">
-        <v>-9.20631895</v>
+        <v>-11.71358519</v>
       </c>
       <c r="B35">
-        <v>16.26063798</v>
+        <v>16.20809556</v>
       </c>
       <c r="C35">
-        <v>-7.12989086</v>
+        <v>-0.29926627</v>
       </c>
     </row>
     <row r="36">
       <c r="A36">
-        <v>11.75617536</v>
+        <v>8.95304878</v>
       </c>
       <c r="B36">
-        <v>16.15065675</v>
+        <v>16.09809571</v>
       </c>
       <c r="C36">
-        <v>-0.9739751</v>
+        <v>-7.7906503</v>
       </c>
     </row>
     <row r="37">
       <c r="A37">
-        <v>-8.11199233</v>
+        <v>-1.3558659</v>
       </c>
       <c r="B37">
-        <v>16.04067551</v>
+        <v>15.98809586</v>
       </c>
       <c r="C37">
-        <v>8.76882601</v>
+        <v>11.93911297</v>
       </c>
     </row>
     <row r="38">
       <c r="A38">
-        <v>0.05898742</v>
+        <v>-7.15022911</v>
       </c>
       <c r="B38">
-        <v>15.93069427</v>
+        <v>15.878096</v>
       </c>
       <c r="C38">
-        <v>-12.09171205</v>
+        <v>-9.83668089</v>
       </c>
     </row>
     <row r="39">
       <c r="A39">
-        <v>8.22078448</v>
+        <v>12.05637896</v>
       </c>
       <c r="B39">
-        <v>15.82071304</v>
+        <v>15.76809615</v>
       </c>
       <c r="C39">
-        <v>9.06221504</v>
+        <v>2.45170762</v>
       </c>
     </row>
     <row r="40">
       <c r="A40">
-        <v>-12.32349083</v>
+        <v>-10.66584786</v>
       </c>
       <c r="B40">
-        <v>15.7107318</v>
+        <v>15.6580963</v>
       </c>
       <c r="C40">
-        <v>-1.14213836</v>
+        <v>6.40809721</v>
       </c>
     </row>
     <row r="41">
       <c r="A41">
-        <v>9.96866634</v>
+        <v>3.57504169</v>
       </c>
       <c r="B41">
-        <v>15.60075057</v>
+        <v>15.54809644</v>
       </c>
       <c r="C41">
-        <v>-7.56586235</v>
+        <v>-12.06133384</v>
       </c>
     </row>
     <row r="42">
       <c r="A42">
-        <v>-2.26423829</v>
+        <v>5.57022233</v>
       </c>
       <c r="B42">
-        <v>15.49076933</v>
+        <v>15.43809659</v>
       </c>
       <c r="C42">
-        <v>12.44625608</v>
+        <v>11.42968927</v>
       </c>
     </row>
     <row r="43">
       <c r="A43">
-        <v>-6.80884453</v>
+        <v>-11.95111391</v>
       </c>
       <c r="B43">
-        <v>15.3807881</v>
+        <v>15.32809674</v>
       </c>
       <c r="C43">
-        <v>-10.81993502</v>
+        <v>-4.71384415</v>
       </c>
     </row>
     <row r="44">
       <c r="A44">
-        <v>12.45590133</v>
+        <v>12.11803292</v>
       </c>
       <c r="B44">
-        <v>15.27080686</v>
+        <v>15.21809688</v>
       </c>
       <c r="C44">
-        <v>3.41364615</v>
+        <v>-4.64357679</v>
       </c>
     </row>
     <row r="45">
       <c r="A45">
-        <v>-11.60518511</v>
+        <v>-5.85591904</v>
       </c>
       <c r="B45">
-        <v>15.16082562</v>
+        <v>15.10809703</v>
       </c>
       <c r="C45">
-        <v>5.95558939</v>
+        <v>11.72406143</v>
       </c>
     </row>
     <row r="46">
       <c r="A46">
-        <v>4.57841945</v>
+        <v>-3.63607455</v>
       </c>
       <c r="B46">
-        <v>15.05084439</v>
+        <v>14.99809718</v>
       </c>
       <c r="C46">
-        <v>-12.34950034</v>
+        <v>-12.72147959</v>
       </c>
     </row>
     <row r="47">
       <c r="A47">
-        <v>5.0129747</v>
+        <v>11.37973502</v>
       </c>
       <c r="B47">
-        <v>14.94086315</v>
+        <v>14.88809732</v>
       </c>
       <c r="C47">
-        <v>12.31424756</v>
+        <v>6.98900486</v>
       </c>
     </row>
     <row r="48">
       <c r="A48">
-        <v>-12.12532896</v>
+        <v>-13.23148329</v>
       </c>
       <c r="B48">
-        <v>14.83088192</v>
+        <v>14.77809747</v>
       </c>
       <c r="C48">
-        <v>-5.74641968</v>
+        <v>2.55649863</v>
       </c>
     </row>
     <row r="49">
       <c r="A49">
-        <v>12.93770803</v>
+        <v>8.10088366</v>
       </c>
       <c r="B49">
-        <v>14.72090068</v>
+        <v>14.66809762</v>
       </c>
       <c r="C49">
-        <v>-3.98883366</v>
+        <v>-10.91891003</v>
       </c>
     </row>
     <row r="50">
       <c r="A50">
-        <v>-6.90542119</v>
+        <v>1.41441998</v>
       </c>
       <c r="B50">
-        <v>14.61091945</v>
+        <v>14.55809776</v>
       </c>
       <c r="C50">
-        <v>11.78287703</v>
+        <v>13.64042542</v>
       </c>
     </row>
     <row r="51">
       <c r="A51">
-        <v>-2.8918819</v>
+        <v>-10.34356836</v>
       </c>
       <c r="B51">
-        <v>14.50093821</v>
+        <v>14.44809791</v>
       </c>
       <c r="C51">
-        <v>-13.46698965</v>
+        <v>-9.17949129</v>
       </c>
     </row>
     <row r="52">
       <c r="A52">
-        <v>11.32285003</v>
+        <v>13.94168198</v>
       </c>
       <c r="B52">
-        <v>14.39095697</v>
+        <v>14.33809806</v>
       </c>
       <c r="C52">
-        <v>8.04322228</v>
+        <v>-0.22010864</v>
       </c>
     </row>
     <row r="53">
       <c r="A53">
-        <v>-13.89442942</v>
+        <v>-10.21302752</v>
       </c>
       <c r="B53">
-        <v>14.28097574</v>
+        <v>14.2280982</v>
       </c>
       <c r="C53">
-        <v>1.73163598</v>
+        <v>9.65687788</v>
       </c>
     </row>
     <row r="54">
       <c r="A54">
-        <v>9.14775706</v>
+        <v>1.01556195</v>
       </c>
       <c r="B54">
-        <v>14.1709945</v>
+        <v>14.11809835</v>
       </c>
       <c r="C54">
-        <v>-10.74716035</v>
+        <v>-14.12968269</v>
       </c>
     </row>
     <row r="55">
       <c r="A55">
-        <v>0.5183245</v>
+        <v>8.86316155</v>
       </c>
       <c r="B55">
-        <v>14.06101327</v>
+        <v>14.0080985</v>
       </c>
       <c r="C55">
-        <v>14.21334745</v>
+        <v>11.19006451</v>
       </c>
     </row>
     <row r="56">
       <c r="A56">
-        <v>-10.0589081</v>
+        <v>-14.19996149</v>
       </c>
       <c r="B56">
-        <v>13.95103203</v>
+        <v>13.89809864</v>
       </c>
       <c r="C56">
-        <v>-10.20720692</v>
+        <v>-2.28121632</v>
       </c>
     </row>
     <row r="57">
       <c r="A57">
-        <v>14.41810799</v>
+        <v>12.09965284</v>
       </c>
       <c r="B57">
-        <v>13.84105079</v>
+        <v>13.78809879</v>
       </c>
       <c r="C57">
-        <v>0.73720755</v>
+        <v>-7.96785623</v>
       </c>
     </row>
     <row r="58">
       <c r="A58">
-        <v>-11.21011038</v>
+        <v>-3.56508329</v>
       </c>
       <c r="B58">
-        <v>13.73106956</v>
+        <v>13.67809894</v>
       </c>
       <c r="C58">
-        <v>9.26235144</v>
+        <v>14.14919752</v>
       </c>
     </row>
     <row r="59">
       <c r="A59">
-        <v>2.02360023</v>
+        <v>-6.97746169</v>
       </c>
       <c r="B59">
-        <v>13.62108832</v>
+        <v>13.56809908</v>
       </c>
       <c r="C59">
-        <v>-14.50417164</v>
+        <v>-12.93142357</v>
       </c>
     </row>
     <row r="60">
       <c r="A60">
-        <v>8.36286672</v>
+        <v>13.97524636</v>
       </c>
       <c r="B60">
-        <v>13.51110709</v>
+        <v>13.45809923</v>
       </c>
       <c r="C60">
-        <v>12.14547016</v>
+        <v>4.85510601</v>
       </c>
     </row>
     <row r="61">
       <c r="A61">
-        <v>-14.46813811</v>
+        <v>-13.67568562</v>
       </c>
       <c r="B61">
-        <v>13.40112585</v>
+        <v>13.34809938</v>
       </c>
       <c r="C61">
-        <v>-3.32908477</v>
+        <v>5.89948014</v>
       </c>
     </row>
     <row r="62">
       <c r="A62">
-        <v>13.00285654</v>
+        <v>6.13905479</v>
       </c>
       <c r="B62">
-        <v>13.29114462</v>
+        <v>13.23809952</v>
       </c>
       <c r="C62">
-        <v>-7.36689871</v>
+        <v>-13.67716079</v>
       </c>
     </row>
     <row r="63">
       <c r="A63">
-        <v>-4.6415937</v>
+        <v>4.74234678</v>
       </c>
       <c r="B63">
-        <v>13.18116338</v>
+        <v>13.12809967</v>
       </c>
       <c r="C63">
-        <v>14.307779</v>
+        <v>14.32351724</v>
       </c>
     </row>
     <row r="64">
       <c r="A64">
-        <v>-6.28190121</v>
+        <v>-13.25520119</v>
       </c>
       <c r="B64">
-        <v>13.07118214</v>
+        <v>13.01809982</v>
       </c>
       <c r="C64">
-        <v>-13.77250575</v>
+        <v>-7.4046417</v>
       </c>
     </row>
     <row r="65">
       <c r="A65">
-        <v>14.02206024</v>
+        <v>14.86685091</v>
       </c>
       <c r="B65">
-        <v>12.96120091</v>
+        <v>12.90809996</v>
       </c>
       <c r="C65">
-        <v>5.94887364</v>
+        <v>-3.51535195</v>
       </c>
     </row>
     <row r="66">
       <c r="A66">
-        <v>-14.44541267</v>
+        <v>-8.63963574</v>
       </c>
       <c r="B66">
-        <v>12.85121967</v>
+        <v>12.79810011</v>
       </c>
       <c r="C66">
-        <v>5.11626874</v>
+        <v>12.71083505</v>
       </c>
     </row>
     <row r="67">
       <c r="A67">
-        <v>7.23860001</v>
+        <v>-2.2285556</v>
       </c>
       <c r="B67">
-        <v>12.74123844</v>
+        <v>12.68810026</v>
       </c>
       <c r="C67">
-        <v>-13.61115399</v>
+        <v>-15.29855064</v>
       </c>
     </row>
     <row r="68">
       <c r="A68">
-        <v>3.87925963</v>
+        <v>12.04672586</v>
       </c>
       <c r="B68">
-        <v>12.6312572</v>
+        <v>12.5781004</v>
       </c>
       <c r="C68">
-        <v>15.01341687</v>
+        <v>9.83197774</v>
       </c>
     </row>
     <row r="69">
       <c r="A69">
-        <v>-13.07643971</v>
+        <v>-15.61248105</v>
       </c>
       <c r="B69">
-        <v>12.52127596</v>
+        <v>12.46810055</v>
       </c>
       <c r="C69">
-        <v>-8.49849237</v>
+        <v>0.89269482</v>
       </c>
     </row>
     <row r="70">
       <c r="A70">
-        <v>15.46928115</v>
+        <v>10.96989371</v>
       </c>
       <c r="B70">
-        <v>12.41129473</v>
+        <v>12.3581007</v>
       </c>
       <c r="C70">
-        <v>-2.58091146</v>
+        <v>-11.2667111</v>
       </c>
     </row>
     <row r="71">
       <c r="A71">
-        <v>-9.71642959</v>
+        <v>-0.48091484</v>
       </c>
       <c r="B71">
-        <v>12.30131349</v>
+        <v>12.24810084</v>
       </c>
       <c r="C71">
-        <v>12.42049445</v>
+        <v>15.80356753</v>
       </c>
     </row>
     <row r="72">
       <c r="A72">
-        <v>-1.23194932</v>
+        <v>-10.37576991</v>
       </c>
       <c r="B72">
-        <v>12.19133226</v>
+        <v>12.13810099</v>
       </c>
       <c r="C72">
-        <v>-15.8067618</v>
+        <v>-12.04200577</v>
       </c>
     </row>
     <row r="73">
       <c r="A73">
-        <v>11.64707237</v>
+        <v>15.86784692</v>
       </c>
       <c r="B73">
-        <v>12.08135102</v>
+        <v>12.02810114</v>
       </c>
       <c r="C73">
-        <v>10.88056353</v>
+        <v>1.88048322</v>
       </c>
     </row>
     <row r="74">
       <c r="A74">
-        <v>-16.02067015</v>
+        <v>-13.03743963</v>
       </c>
       <c r="B74">
-        <v>11.97136979</v>
+        <v>11.91810128</v>
       </c>
       <c r="C74">
-        <v>-0.15631212</v>
+        <v>9.37998026</v>
       </c>
     </row>
     <row r="75">
       <c r="A75">
-        <v>11.97943048</v>
+        <v>3.29385388</v>
       </c>
       <c r="B75">
-        <v>11.86138855</v>
+        <v>11.80810143</v>
       </c>
       <c r="C75">
-        <v>-10.76107369</v>
+        <v>-15.80250826</v>
       </c>
     </row>
     <row r="76">
       <c r="A76">
-        <v>-1.57207189</v>
+        <v>8.28646631</v>
       </c>
       <c r="B76">
-        <v>11.75140731</v>
+        <v>11.69810158</v>
       </c>
       <c r="C76">
-        <v>16.10692448</v>
+        <v>13.94592756</v>
       </c>
     </row>
     <row r="77">
       <c r="A77">
-        <v>-9.76850325</v>
+        <v>-15.60592313</v>
       </c>
       <c r="B77">
-        <v>11.64142608</v>
+        <v>11.58810172</v>
       </c>
       <c r="C77">
-        <v>-13.00205919</v>
+        <v>-4.70861568</v>
       </c>
     </row>
     <row r="78">
       <c r="A78">
-        <v>16.06259215</v>
+        <v>14.75790605</v>
       </c>
       <c r="B78">
-        <v>11.53144484</v>
+        <v>11.47810187</v>
       </c>
       <c r="C78">
-        <v>3.00315054</v>
+        <v>-7.1033363</v>
       </c>
     </row>
     <row r="79">
       <c r="A79">
-        <v>-13.9380745</v>
+        <v>-6.11221687</v>
       </c>
       <c r="B79">
-        <v>11.42146361</v>
+        <v>11.36810202</v>
       </c>
       <c r="C79">
-        <v>8.67641909</v>
+        <v>15.27766545</v>
       </c>
     </row>
     <row r="80">
       <c r="A80">
-        <v>4.43710146</v>
+        <v>-5.83961142</v>
       </c>
       <c r="B80">
-        <v>11.31148237</v>
+        <v>11.25810216</v>
       </c>
       <c r="C80">
-        <v>-15.88592135</v>
+        <v>-15.46460714</v>
       </c>
     </row>
     <row r="81">
       <c r="A81">
-        <v>7.49287152</v>
+        <v>14.81852034</v>
       </c>
       <c r="B81">
-        <v>11.20150113</v>
+        <v>11.14810231</v>
       </c>
       <c r="C81">
-        <v>14.7777958</v>
+        <v>7.49208047</v>
       </c>
     </row>
     <row r="82">
       <c r="A82">
-        <v>-15.57636221</v>
+        <v>-16.05814277</v>
       </c>
       <c r="B82">
-        <v>11.0915199</v>
+        <v>11.03810246</v>
       </c>
       <c r="C82">
-        <v>-5.86132465</v>
+        <v>4.50514651</v>
       </c>
     </row>
     <row r="83">
       <c r="A83">
-        <v>15.51232923</v>
+        <v>8.83572013</v>
       </c>
       <c r="B83">
-        <v>10.98153866</v>
+        <v>10.9281026</v>
       </c>
       <c r="C83">
-        <v>-6.2268331</v>
+        <v>-14.23048219</v>
       </c>
     </row>
     <row r="84">
       <c r="A84">
-        <v>-7.26318208</v>
+        <v>3.11054298</v>
       </c>
       <c r="B84">
-        <v>10.87155743</v>
+        <v>10.81810275</v>
       </c>
       <c r="C84">
-        <v>15.13457714</v>
+        <v>16.53158115</v>
       </c>
     </row>
     <row r="85">
       <c r="A85">
-        <v>-4.88812033</v>
+        <v>-13.51674172</v>
       </c>
       <c r="B85">
-        <v>10.76157619</v>
+        <v>10.7081029</v>
       </c>
       <c r="C85">
-        <v>-16.13365295</v>
+        <v>-10.13085513</v>
       </c>
     </row>
     <row r="86">
       <c r="A86">
-        <v>14.56244022</v>
+        <v>16.87901476</v>
       </c>
       <c r="B86">
-        <v>10.65159496</v>
+        <v>10.59810304</v>
       </c>
       <c r="C86">
-        <v>8.63011354</v>
+        <v>-1.66705505</v>
       </c>
     </row>
     <row r="87">
       <c r="A87">
-        <v>-16.63469467</v>
+        <v>-11.36552387</v>
       </c>
       <c r="B87">
-        <v>10.54161372</v>
+        <v>10.48810319</v>
       </c>
       <c r="C87">
-        <v>3.48730749</v>
+        <v>12.6816623</v>
       </c>
     </row>
     <row r="88">
       <c r="A88">
-        <v>9.94975186</v>
+        <v>-0.18648987</v>
       </c>
       <c r="B88">
-        <v>10.43163248</v>
+        <v>10.37810334</v>
       </c>
       <c r="C88">
-        <v>-13.8630257</v>
+        <v>-17.09561911</v>
       </c>
     </row>
     <row r="89">
       <c r="A89">
-        <v>2.03563367</v>
+        <v>11.73074565</v>
       </c>
       <c r="B89">
-        <v>10.32165125</v>
+        <v>10.26810349</v>
       </c>
       <c r="C89">
-        <v>17.00940067</v>
+        <v>12.5281945</v>
       </c>
     </row>
     <row r="90">
       <c r="A90">
-        <v>-13.04058563</v>
+        <v>-17.17770183</v>
       </c>
       <c r="B90">
-        <v>10.21167001</v>
+        <v>10.15810363</v>
       </c>
       <c r="C90">
-        <v>-11.21003666</v>
+        <v>-1.31889742</v>
       </c>
     </row>
     <row r="91">
       <c r="A91">
-        <v>17.25279583</v>
+        <v>13.60787193</v>
       </c>
       <c r="B91">
-        <v>10.10168878</v>
+        <v>10.04810378</v>
       </c>
       <c r="C91">
-        <v>-0.54490357</v>
+        <v>-10.67058723</v>
       </c>
     </row>
     <row r="92">
       <c r="A92">
-        <v>-12.39932544</v>
+        <v>-2.83651289</v>
       </c>
       <c r="B92">
-        <v>9.99170754</v>
+        <v>9.93810393</v>
       </c>
       <c r="C92">
-        <v>12.10051689</v>
+        <v>17.12274175</v>
       </c>
     </row>
     <row r="93">
       <c r="A93">
-        <v>0.97261689</v>
+        <v>-9.50882178</v>
       </c>
       <c r="B93">
-        <v>9.88172631</v>
+        <v>9.82810407</v>
       </c>
       <c r="C93">
-        <v>-17.361034</v>
+        <v>-14.59420017</v>
       </c>
     </row>
     <row r="94">
       <c r="A94">
-        <v>11.04931786</v>
+        <v>16.92941739</v>
       </c>
       <c r="B94">
-        <v>9.77174507</v>
+        <v>9.71810422</v>
       </c>
       <c r="C94">
-        <v>13.50650114</v>
+        <v>4.35353619</v>
       </c>
     </row>
     <row r="95">
       <c r="A95">
-        <v>-17.33143833</v>
+        <v>-15.47755909</v>
       </c>
       <c r="B95">
-        <v>9.66176383</v>
+        <v>9.60810437</v>
       </c>
       <c r="C95">
-        <v>-2.50430927</v>
+        <v>8.25405931</v>
       </c>
     </row>
     <row r="96">
       <c r="A96">
-        <v>14.52107516</v>
+        <v>5.85703518</v>
       </c>
       <c r="B96">
-        <v>9.5517826</v>
+        <v>9.49810451</v>
       </c>
       <c r="C96">
-        <v>-9.89453513</v>
+        <v>-16.59762482</v>
       </c>
     </row>
     <row r="97">
       <c r="A97">
-        <v>-4.03731476</v>
+        <v>6.91581237</v>
       </c>
       <c r="B97">
-        <v>9.44180136</v>
+        <v>9.38810466</v>
       </c>
       <c r="C97">
-        <v>17.16253118</v>
+        <v>16.24915475</v>
       </c>
     </row>
     <row r="98">
       <c r="A98">
-        <v>-8.6447007</v>
+        <v>-16.12848461</v>
       </c>
       <c r="B98">
-        <v>9.33182013</v>
+        <v>9.27810481</v>
       </c>
       <c r="C98">
-        <v>-15.43328491</v>
+        <v>-7.33408177</v>
       </c>
     </row>
     <row r="99">
       <c r="A99">
-        <v>16.85405333</v>
+        <v>16.90110255</v>
       </c>
       <c r="B99">
-        <v>9.22183889</v>
+        <v>9.16810495</v>
       </c>
       <c r="C99">
-        <v>5.55864856</v>
+        <v>-5.50441498</v>
       </c>
     </row>
     <row r="100">
       <c r="A100">
-        <v>-16.23418507</v>
+        <v>-8.77186795</v>
       </c>
       <c r="B100">
-        <v>9.11185765</v>
+        <v>9.0581051</v>
       </c>
       <c r="C100">
-        <v>7.30926023</v>
+        <v>15.52433782</v>
       </c>
     </row>
     <row r="101">
       <c r="A101">
-        <v>7.05531574</v>
+        <v>-4.03093412</v>
       </c>
       <c r="B101">
-        <v>9.00187642</v>
+        <v>8.94810525</v>
       </c>
       <c r="C101">
-        <v>-16.40697232</v>
+        <v>-17.42650231</v>
       </c>
     </row>
     <row r="102">
       <c r="A102">
-        <v>5.898493</v>
+        <v>14.78873105</v>
       </c>
       <c r="B102">
-        <v>8.89189518</v>
+        <v>8.83810539</v>
       </c>
       <c r="C102">
-        <v>16.91573174</v>
+        <v>10.15782097</v>
       </c>
     </row>
     <row r="103">
       <c r="A103">
-        <v>-15.82347987</v>
+        <v>-17.8195048</v>
       </c>
       <c r="B103">
-        <v>8.78191395</v>
+        <v>8.72810554</v>
       </c>
       <c r="C103">
-        <v>-8.5144273</v>
+        <v>2.50707446</v>
       </c>
     </row>
     <row r="104">
       <c r="A104">
-        <v>17.47085862</v>
+        <v>11.47971665</v>
       </c>
       <c r="B104">
-        <v>8.67193271</v>
+        <v>8.61810569</v>
       </c>
       <c r="C104">
-        <v>-4.42342425</v>
+        <v>-13.92639078</v>
       </c>
     </row>
     <row r="105">
       <c r="A105">
-        <v>-9.92331564</v>
+        <v>0.94507719</v>
       </c>
       <c r="B105">
-        <v>8.56195148</v>
+        <v>8.50810583</v>
       </c>
       <c r="C105">
-        <v>15.10697831</v>
+        <v>18.07536899</v>
       </c>
     </row>
     <row r="106">
       <c r="A106">
-        <v>-2.89573064</v>
+        <v>-12.94318698</v>
       </c>
       <c r="B106">
-        <v>8.45197024</v>
+        <v>8.39810598</v>
       </c>
       <c r="C106">
-        <v>-17.89354473</v>
+        <v>-12.72578983</v>
       </c>
     </row>
     <row r="107">
       <c r="A107">
-        <v>14.26205623</v>
+        <v>18.19050953</v>
       </c>
       <c r="B107">
-        <v>8.341989</v>
+        <v>8.28810613</v>
       </c>
       <c r="C107">
-        <v>11.26964825</v>
+        <v>0.6423861</v>
       </c>
     </row>
     <row r="108">
       <c r="A108">
-        <v>-18.17887292</v>
+        <v>-13.88484097</v>
       </c>
       <c r="B108">
-        <v>8.23200777</v>
+        <v>8.17810627</v>
       </c>
       <c r="C108">
-        <v>1.32763979</v>
+        <v>11.84608665</v>
       </c>
     </row>
     <row r="109">
       <c r="A109">
-        <v>12.54153859</v>
+        <v>2.24232366</v>
       </c>
       <c r="B109">
-        <v>8.12202653</v>
+        <v>8.06810642</v>
       </c>
       <c r="C109">
-        <v>-13.29445354</v>
+        <v>-18.16253406</v>
       </c>
     </row>
     <row r="110">
       <c r="A110">
-        <v>-0.26817538</v>
+        <v>10.64309733</v>
       </c>
       <c r="B110">
-        <v>8.0120453</v>
+        <v>7.95810657</v>
       </c>
       <c r="C110">
-        <v>18.32307868</v>
+        <v>14.94633798</v>
       </c>
     </row>
     <row r="111">
       <c r="A111">
-        <v>-12.21101616</v>
+        <v>-17.99027003</v>
       </c>
       <c r="B111">
-        <v>7.90206406</v>
+        <v>7.84810671</v>
       </c>
       <c r="C111">
-        <v>-13.7276534</v>
+        <v>-3.84153682</v>
       </c>
     </row>
     <row r="112">
       <c r="A112">
-        <v>18.32358883</v>
+        <v>15.90051225</v>
       </c>
       <c r="B112">
-        <v>7.79208282</v>
+        <v>7.73810686</v>
       </c>
       <c r="C112">
-        <v>1.87870642</v>
+        <v>-9.3432014</v>
       </c>
     </row>
     <row r="113">
       <c r="A113">
-        <v>-14.81731522</v>
+        <v>-5.42673542</v>
       </c>
       <c r="B113">
-        <v>7.68210159</v>
+        <v>7.62810701</v>
       </c>
       <c r="C113">
-        <v>11.01964087</v>
+        <v>17.67378076</v>
       </c>
     </row>
     <row r="114">
       <c r="A114">
-        <v>3.49072241</v>
+        <v>-7.95628146</v>
       </c>
       <c r="B114">
-        <v>7.57212035</v>
+        <v>7.51810715</v>
       </c>
       <c r="C114">
-        <v>-18.17904977</v>
+        <v>-16.73844826</v>
       </c>
     </row>
     <row r="115">
       <c r="A115">
-        <v>9.72921067</v>
+        <v>17.21437051</v>
       </c>
       <c r="B115">
-        <v>7.46213912</v>
+        <v>7.4081073</v>
       </c>
       <c r="C115">
-        <v>15.80059934</v>
+        <v>6.98465419</v>
       </c>
     </row>
     <row r="116">
       <c r="A116">
-        <v>-17.88934494</v>
+        <v>-17.45216574</v>
       </c>
       <c r="B116">
-        <v>7.35215788</v>
+        <v>7.29810745</v>
       </c>
       <c r="C116">
-        <v>-5.09088521</v>
+        <v>6.4930377</v>
       </c>
     </row>
     <row r="117">
       <c r="A117">
-        <v>16.6684244</v>
+        <v>8.5021693</v>
       </c>
       <c r="B117">
-        <v>7.24217665</v>
+        <v>7.18810759</v>
       </c>
       <c r="C117">
-        <v>-8.34952127</v>
+        <v>-16.61457873</v>
       </c>
     </row>
     <row r="118">
       <c r="A118">
-        <v>-6.66586587</v>
+        <v>4.96489778</v>
       </c>
       <c r="B118">
-        <v>7.13219541</v>
+        <v>7.07810774</v>
       </c>
       <c r="C118">
-        <v>17.45560142</v>
+        <v>18.03469381</v>
       </c>
     </row>
     <row r="119">
       <c r="A119">
-        <v>-6.89119946</v>
+        <v>-15.87816326</v>
       </c>
       <c r="B119">
-        <v>7.02221417</v>
+        <v>6.96810789</v>
       </c>
       <c r="C119">
-        <v>-17.41263559</v>
+        <v>-9.9664138</v>
       </c>
     </row>
     <row r="120">
       <c r="A120">
-        <v>16.88018556</v>
+        <v>18.48013634</v>
       </c>
       <c r="B120">
-        <v>6.91223294</v>
+        <v>6.85810803</v>
       </c>
       <c r="C120">
-        <v>8.20246128</v>
+        <v>-3.3839201</v>
       </c>
     </row>
     <row r="121">
       <c r="A121">
-        <v>-18.02608</v>
+        <v>-11.36489111</v>
       </c>
       <c r="B121">
-        <v>6.8022517</v>
+        <v>6.74810818</v>
       </c>
       <c r="C121">
-        <v>5.36561381</v>
+        <v>15.01007282</v>
       </c>
     </row>
     <row r="122">
       <c r="A122">
-        <v>9.68771</v>
+        <v>-1.76269135</v>
       </c>
       <c r="B122">
-        <v>6.69227047</v>
+        <v>6.63810833</v>
       </c>
       <c r="C122">
-        <v>-16.1666877</v>
+        <v>-18.78372799</v>
       </c>
     </row>
     <row r="123">
       <c r="A123">
-        <v>3.78477874</v>
+        <v>14.01640896</v>
       </c>
       <c r="B123">
-        <v>6.58228923</v>
+        <v>6.52810847</v>
       </c>
       <c r="C123">
-        <v>18.50267328</v>
+        <v>12.68558551</v>
       </c>
     </row>
     <row r="124">
       <c r="A124">
-        <v>-15.319896</v>
+        <v>-18.94188047</v>
       </c>
       <c r="B124">
-        <v>6.47230799</v>
+        <v>6.41810862</v>
       </c>
       <c r="C124">
-        <v>-11.10900607</v>
+        <v>0.11421914</v>
       </c>
     </row>
     <row r="125">
       <c r="A125">
-        <v>18.83745697</v>
+        <v>13.91706863</v>
       </c>
       <c r="B125">
-        <v>6.36232676</v>
+        <v>6.30810877</v>
       </c>
       <c r="C125">
-        <v>-2.1612527</v>
+        <v>-12.90437773</v>
       </c>
     </row>
     <row r="126">
       <c r="A126">
-        <v>-12.45421013</v>
+        <v>-1.54817929</v>
       </c>
       <c r="B126">
-        <v>6.25234552</v>
+        <v>6.19810891</v>
       </c>
       <c r="C126">
-        <v>14.34575985</v>
+        <v>18.95221852</v>
       </c>
     </row>
     <row r="127">
       <c r="A127">
-        <v>-0.50803133</v>
+        <v>-11.68223163</v>
       </c>
       <c r="B127">
-        <v>6.14236429</v>
+        <v>6.08810906</v>
       </c>
       <c r="C127">
-        <v>-19.02664619</v>
+        <v>-15.048601</v>
       </c>
     </row>
     <row r="128">
       <c r="A128">
-        <v>13.25134283</v>
+        <v>18.81360532</v>
       </c>
       <c r="B128">
-        <v>6.03238305</v>
+        <v>5.97810921</v>
       </c>
       <c r="C128">
-        <v>13.71175655</v>
+        <v>3.21099133</v>
       </c>
     </row>
     <row r="129">
       <c r="A129">
-        <v>-19.06766706</v>
+        <v>-16.0702278</v>
       </c>
       <c r="B129">
-        <v>5.92240182</v>
+        <v>5.86810935</v>
       </c>
       <c r="C129">
-        <v>-1.16156348</v>
+        <v>10.35920224</v>
       </c>
     </row>
     <row r="130">
       <c r="A130">
-        <v>14.87075586</v>
+        <v>4.86062516</v>
       </c>
       <c r="B130">
-        <v>5.81242058</v>
+        <v>5.7581095</v>
       </c>
       <c r="C130">
-        <v>-12.04476596</v>
+        <v>-18.52615713</v>
       </c>
     </row>
     <row r="131">
       <c r="A131">
-        <v>-2.83399754</v>
+        <v>8.94542408</v>
       </c>
       <c r="B131">
-        <v>5.70243934</v>
+        <v>5.64810965</v>
       </c>
       <c r="C131">
-        <v>18.95918362</v>
+        <v>16.97286792</v>
       </c>
     </row>
     <row r="132">
       <c r="A132">
-        <v>-10.73514145</v>
+        <v>-18.09124701</v>
       </c>
       <c r="B132">
-        <v>5.59245811</v>
+        <v>5.53810979</v>
       </c>
       <c r="C132">
-        <v>-15.92109137</v>
+        <v>-6.48352692</v>
       </c>
     </row>
     <row r="133">
       <c r="A133">
-        <v>18.70111398</v>
+        <v>17.74839562</v>
       </c>
       <c r="B133">
-        <v>5.48247687</v>
+        <v>5.42810994</v>
       </c>
       <c r="C133">
-        <v>4.49564047</v>
+        <v>-7.45185047</v>
       </c>
     </row>
     <row r="134">
       <c r="A134">
-        <v>-16.85350932</v>
+        <v>-8.06629774</v>
       </c>
       <c r="B134">
-        <v>5.37249564</v>
+        <v>5.31811009</v>
       </c>
       <c r="C134">
-        <v>9.33249774</v>
+        <v>17.51149753</v>
       </c>
     </row>
     <row r="135">
       <c r="A135">
-        <v>6.13288285</v>
+        <v>-5.89016211</v>
       </c>
       <c r="B135">
-        <v>5.2625144</v>
+        <v>5.20811023</v>
       </c>
       <c r="C135">
-        <v>-18.29463556</v>
+        <v>-18.38971392</v>
       </c>
     </row>
     <row r="136">
       <c r="A136">
-        <v>7.84769638</v>
+        <v>16.79076257</v>
       </c>
       <c r="B136">
-        <v>5.15253317</v>
+        <v>5.09811038</v>
       </c>
       <c r="C136">
-        <v>17.65970168</v>
+        <v>9.59580965</v>
       </c>
     </row>
     <row r="137">
       <c r="A137">
-        <v>-17.74217931</v>
+        <v>-18.89081927</v>
       </c>
       <c r="B137">
-        <v>5.04255193</v>
+        <v>4.98811053</v>
       </c>
       <c r="C137">
-        <v>-7.73225345</v>
+        <v>4.27266904</v>
       </c>
     </row>
     <row r="138">
       <c r="A138">
-        <v>18.3323808</v>
+        <v>11.05931937</v>
       </c>
       <c r="B138">
-        <v>4.93257069</v>
+        <v>4.87811067</v>
       </c>
       <c r="C138">
-        <v>-6.29234142</v>
+        <v>-15.93409839</v>
       </c>
     </row>
     <row r="139">
       <c r="A139">
-        <v>-9.28053544</v>
+        <v>2.61220698</v>
       </c>
       <c r="B139">
-        <v>4.82258946</v>
+        <v>4.76811082</v>
       </c>
       <c r="C139">
-        <v>17.04741308</v>
+        <v>19.24685673</v>
       </c>
     </row>
     <row r="140">
       <c r="A140">
-        <v>-4.67868225</v>
+        <v>-14.94772411</v>
       </c>
       <c r="B140">
-        <v>4.71260822</v>
+        <v>4.65811097</v>
       </c>
       <c r="C140">
-        <v>-18.86534538</v>
+        <v>-12.44457898</v>
       </c>
     </row>
     <row r="141">
       <c r="A141">
-        <v>16.21521411</v>
+        <v>19.45416531</v>
       </c>
       <c r="B141">
-        <v>4.60262699</v>
+        <v>4.54811111</v>
       </c>
       <c r="C141">
-        <v>10.76488068</v>
+        <v>-0.92202894</v>
       </c>
     </row>
     <row r="142">
       <c r="A142">
-        <v>-19.25353708</v>
+        <v>-13.73994248</v>
       </c>
       <c r="B142">
-        <v>4.49264575</v>
+        <v>4.43811126</v>
       </c>
       <c r="C142">
-        <v>3.01951058</v>
+        <v>13.83897211</v>
       </c>
     </row>
     <row r="143">
       <c r="A143">
-        <v>12.1729209</v>
+        <v>0.78430707</v>
       </c>
       <c r="B143">
-        <v>4.38266451</v>
+        <v>4.32811141</v>
       </c>
       <c r="C143">
-        <v>-15.25163101</v>
+        <v>-19.51031302</v>
       </c>
     </row>
     <row r="144">
       <c r="A144">
-        <v>1.32805255</v>
+        <v>12.61622854</v>
       </c>
       <c r="B144">
-        <v>4.27268328</v>
+        <v>4.21811155</v>
       </c>
       <c r="C144">
-        <v>19.49308734</v>
+        <v>14.93446726</v>
       </c>
     </row>
     <row r="145">
       <c r="A145">
-        <v>-14.16383545</v>
+        <v>-19.41412126</v>
       </c>
       <c r="B145">
-        <v>4.16270204</v>
+        <v>4.1081117</v>
       </c>
       <c r="C145">
-        <v>-13.49287504</v>
+        <v>-2.49305313</v>
       </c>
     </row>
     <row r="146">
       <c r="A146">
-        <v>19.5813539</v>
+        <v>16.01800973</v>
       </c>
       <c r="B146">
-        <v>4.05272081</v>
+        <v>3.99811185</v>
       </c>
       <c r="C146">
-        <v>0.38214311</v>
+        <v>-11.28886469</v>
       </c>
     </row>
     <row r="147">
       <c r="A147">
-        <v>-14.71365157</v>
+        <v>-4.19038834</v>
       </c>
       <c r="B147">
-        <v>3.94273957</v>
+        <v>3.88811199</v>
       </c>
       <c r="C147">
-        <v>12.96006412</v>
+        <v>19.16567846</v>
       </c>
     </row>
     <row r="148">
       <c r="A148">
-        <v>2.09731992</v>
+        <v>-9.86715965</v>
       </c>
       <c r="B148">
-        <v>3.83275834</v>
+        <v>3.77811214</v>
       </c>
       <c r="C148">
-        <v>-19.51694681</v>
+        <v>-16.98131412</v>
       </c>
     </row>
     <row r="149">
       <c r="A149">
-        <v>11.64955125</v>
+        <v>18.76634267</v>
       </c>
       <c r="B149">
-        <v>3.7227771</v>
+        <v>3.66811229</v>
       </c>
       <c r="C149">
-        <v>15.82494506</v>
+        <v>5.86253658</v>
       </c>
     </row>
     <row r="150">
       <c r="A150">
-        <v>-19.29974355</v>
+        <v>-17.81609373</v>
       </c>
       <c r="B150">
-        <v>3.61279586</v>
+        <v>3.55811243</v>
       </c>
       <c r="C150">
-        <v>-3.80363049</v>
+        <v>8.36221502</v>
       </c>
     </row>
     <row r="151">
       <c r="A151">
-        <v>16.8173261</v>
+        <v>7.49588407</v>
       </c>
       <c r="B151">
-        <v>3.50281463</v>
+        <v>3.44811258</v>
       </c>
       <c r="C151">
-        <v>-10.24245246</v>
+        <v>-18.21873326</v>
       </c>
     </row>
     <row r="152">
       <c r="A152">
-        <v>-5.48725427</v>
+        <v>6.78586236</v>
       </c>
       <c r="B152">
-        <v>3.39283339</v>
+        <v>3.33811273</v>
       </c>
       <c r="C152">
-        <v>18.93089333</v>
+        <v>18.51510398</v>
       </c>
     </row>
     <row r="153">
       <c r="A153">
-        <v>-8.74976052</v>
+        <v>-17.52671164</v>
       </c>
       <c r="B153">
-        <v>3.28285216</v>
+        <v>3.22811287</v>
       </c>
       <c r="C153">
-        <v>-17.68232373</v>
+        <v>-9.0770957</v>
       </c>
     </row>
     <row r="154">
       <c r="A154">
-        <v>18.41281026</v>
+        <v>19.07220648</v>
       </c>
       <c r="B154">
-        <v>3.17287092</v>
+        <v>3.11811302</v>
       </c>
       <c r="C154">
-        <v>7.1345153</v>
+        <v>-5.15056416</v>
       </c>
     </row>
     <row r="155">
       <c r="A155">
-        <v>-18.41249977</v>
+        <v>-10.59322912</v>
       </c>
       <c r="B155">
-        <v>3.06288968</v>
+        <v>3.00811317</v>
       </c>
       <c r="C155">
-        <v>7.1832137</v>
+        <v>16.69535121</v>
       </c>
     </row>
     <row r="156">
       <c r="A156">
-        <v>8.73199885</v>
+        <v>-3.46930929</v>
       </c>
       <c r="B156">
-        <v>2.95290845</v>
+        <v>2.89811331</v>
       </c>
       <c r="C156">
-        <v>-17.74915569</v>
+        <v>-19.48242367</v>
       </c>
     </row>
     <row r="157">
       <c r="A157">
-        <v>5.55519765</v>
+        <v>15.73089685</v>
       </c>
       <c r="B157">
-        <v>2.84292721</v>
+        <v>2.78811346</v>
       </c>
       <c r="C157">
-        <v>19.00151425</v>
+        <v>12.03184556</v>
       </c>
     </row>
     <row r="158">
       <c r="A158">
-        <v>-16.94480972</v>
+        <v>-19.74198354</v>
       </c>
       <c r="B158">
-        <v>2.73294598</v>
+        <v>2.67811361</v>
       </c>
       <c r="C158">
-        <v>-10.26666596</v>
+        <v>1.75550373</v>
       </c>
     </row>
     <row r="159">
       <c r="A159">
-        <v>19.44418155</v>
+        <v>13.38111648</v>
       </c>
       <c r="B159">
-        <v>2.62296474</v>
+        <v>2.56811375</v>
       </c>
       <c r="C159">
-        <v>-3.8786415</v>
+        <v>-14.64071424</v>
       </c>
     </row>
     <row r="160">
       <c r="A160">
-        <v>-11.72596485</v>
+        <v>0.02285756</v>
       </c>
       <c r="B160">
-        <v>2.51298351</v>
+        <v>2.4581139</v>
       </c>
       <c r="C160">
-        <v>16.00583213</v>
+        <v>19.84835393</v>
       </c>
     </row>
     <row r="161">
       <c r="A161">
-        <v>-2.16690914</v>
+        <v>-13.43322941</v>
       </c>
       <c r="B161">
-        <v>2.40300227</v>
+        <v>2.34811405</v>
       </c>
       <c r="C161">
-        <v>-19.73651653</v>
+        <v>-14.62992509</v>
       </c>
     </row>
     <row r="162">
       <c r="A162">
-        <v>14.93941317</v>
+        <v>19.80026624</v>
       </c>
       <c r="B162">
-        <v>2.29302103</v>
+        <v>2.23811419</v>
       </c>
       <c r="C162">
-        <v>13.09793834</v>
+        <v>1.71473074</v>
       </c>
     </row>
     <row r="163">
       <c r="A163">
-        <v>-19.8757705</v>
+        <v>-15.76796178</v>
       </c>
       <c r="B163">
-        <v>2.1830398</v>
+        <v>2.12811434</v>
       </c>
       <c r="C163">
-        <v>0.43368667</v>
+        <v>12.11785916</v>
       </c>
     </row>
     <row r="164">
       <c r="A164">
-        <v>14.37132616</v>
+        <v>3.44329184</v>
       </c>
       <c r="B164">
-        <v>2.07305856</v>
+        <v>2.01811449</v>
       </c>
       <c r="C164">
-        <v>-13.75381447</v>
+        <v>-19.59772832</v>
       </c>
     </row>
     <row r="165">
       <c r="A165">
-        <v>-1.30713302</v>
+        <v>10.70493282</v>
       </c>
       <c r="B165">
-        <v>1.96307733</v>
+        <v>1.90811463</v>
       </c>
       <c r="C165">
-        <v>19.86045646</v>
+        <v>16.78581281</v>
       </c>
     </row>
     <row r="166">
       <c r="A166">
-        <v>-12.45830077</v>
+        <v>-19.24202624</v>
       </c>
       <c r="B166">
-        <v>1.85309609</v>
+        <v>1.79811478</v>
       </c>
       <c r="C166">
-        <v>-15.53566146</v>
+        <v>-5.14890371</v>
       </c>
     </row>
   </sheetData>

</xml_diff>